<commit_message>
Arricchiti abstract padri F24 (284) e IVA (294)
ID 284 'Pagare con F24': abstract menziona varianti semplificato/ELIDE/accise/EP/cumulativo
+ parole chiave includono tutti i modelli archiviati per coprire ricerca utente.
ID 294 'Versamenti IVA': abstract include sia liquidazione periodica sia acconto IVA dicembre.
</commit_message>
<xml_diff>
--- a/DB_Schede_Import_CardSorting.xlsx
+++ b/DB_Schede_Import_CardSorting.xlsx
@@ -9615,7 +9615,7 @@
       </c>
       <c r="N196" t="inlineStr">
         <is>
-          <t>Pagare con il modello F24 ordinario: strumento unificato per il versamento di tributi, contributi e premi (IRPEF, IVA, INPS, INAIL) con possibilità di compensazione tra crediti e debiti.</t>
+          <t>Pagare con il modello F24 come contribuente: strumento unificato per versare tributi, contributi e premi (IRPEF, IVA, INPS), con varianti semplificato, ELIDE, accise, enti pubblici e cumulativo per intermediari.</t>
         </is>
       </c>
     </row>
@@ -10103,7 +10103,7 @@
       </c>
       <c r="N205" t="inlineStr">
         <is>
-          <t>Versare l'IVA periodica come impresa: liquidazione e versamento mensile (entro il 16 del mese successivo) o trimestrale (entro il 16 del secondo mese), tramite F24.</t>
+          <t>Versare l'IVA come impresa: liquidazione periodica mensile (entro il 16 del mese successivo) o trimestrale, più acconto IVA entro il 27 dicembre tramite modello F24.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
DB update: 46 schede compilate (richiesta Giulia) + archiviato ID 183 duplicato 770/2026
- 47 schede 'Da verificare/Da classificare' completate con titolo TO-BE, macro/sotto, abstract, parole chiave, use case, life event
- ID 183 archiviato (duplicato di ID 173 - Modello 770/2026)
- Le altre 46 marcate come 'Attiva'
- DB Card Sorting rigenerato con schede attive aggiornate
</commit_message>
<xml_diff>
--- a/DB_Schede_Import_CardSorting.xlsx
+++ b/DB_Schede_Import_CardSorting.xlsx
@@ -661,7 +661,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Comunicazione di irregolarità</t>
+          <t>Rispondere a una comunicazione di irregolarità dell'Agenzia delle Entrate</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -672,10 +672,40 @@
       <c r="D5" t="inlineStr">
         <is>
           <t>Accertamenti e regolarizzazioni</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Rispondere a una comunicazione di irregolarità dell'Agenzia delle Entrate</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Controlli fiscali e contenziosi</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Controlli automatici</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Life events — Adempimenti fiscali / risposta a comunicazioni</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Rispondere a una comunicazione di irregolarità come contribuente: verificare l'esito della liquidazione automatica della dichiarazione, sanare gli errori o presentare chiarimenti entro 30 giorni per evitare l'iscrizione a ruolo.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -735,7 +765,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Ravvedimento</t>
+          <t>Regolarizzare la propria posizione fiscale con il ravvedimento operoso</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -746,10 +776,40 @@
       <c r="D7" t="inlineStr">
         <is>
           <t>Accertamenti e regolarizzazioni</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Regolarizzare la propria posizione fiscale con il ravvedimento operoso</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Controlli fiscali e contenziosi</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Controlli automatici</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti ricorrenti</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Regolarizzare spontaneamente errori o omissioni fiscali come contribuente: sanare violazioni pagando l'imposta dovuta con interessi e sanzioni ridotte, prima che l'Agenzia notifichi accertamenti.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -950,7 +1010,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Agevolazioni per persone con disabilità</t>
+          <t>Ottenere le agevolazioni fiscali per persone con disabilità</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -961,6 +1021,16 @@
       <c r="D12" t="inlineStr">
         <is>
           <t>Agevolazioni</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Ottenere le agevolazioni fiscali per persone con disabilità</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -970,19 +1040,14 @@
           <t>Agevolazioni per persone con disabilità</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Agevolazioni fiscali</t>
-        </is>
-      </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Family — Eventi familiari / Famiglia</t>
+          <t>Life events — Disabilità / assistenza familiare</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Sezione dedicata alle agevolazioni fiscali per le persone con disabilità: detrazioni, IVA agevolata, esenzioni e servizi dedicati.</t>
+          <t>Ottenere le agevolazioni fiscali come persona con disabilità o familiare: IVA agevolata su veicoli e ausili, detrazioni per spese sanitarie, agevolazioni sulle successioni e sull'imposta di registro.</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2316,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Riqualificazione energetica</t>
+          <t>Richiedere le detrazioni per interventi di riqualificazione energetica (Ecobonus)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2262,10 +2327,40 @@
       <c r="D40" t="inlineStr">
         <is>
           <t>Agevolazioni</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Richiedere le detrazioni per interventi di riqualificazione energetica (Ecobonus)</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Ottenere bonus e agevolazioni</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Agevolazioni casa e ristrutturazioni</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Property purchase / renovation — Casa</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Richiedere le detrazioni per interventi di riqualificazione energetica come proprietario o inquilino: coibentazione, infissi, pannelli solari, caldaie a condensazione, con recupero fiscale in dichiarazione.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -3801,7 +3896,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Comunicare i trasferimenti da e verso l'estero (monitoraggio fiscale)</t>
+          <t>Comunicare i dati dei trasferimenti da/verso l'estero come intermediario finanziario</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3816,7 +3911,12 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Comunicare i trasferimenti da e verso l'estero (monitoraggio fiscale)</t>
+          <t>Comunicare i dati dei trasferimenti da/verso l'estero come intermediario finanziario</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G75" t="inlineStr"/>
@@ -3843,12 +3943,12 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>Regular Business Operations — Gestione attività / Adempimenti ricorrenti</t>
+          <t>Regular Business Operations — Comunicazioni ricorrenti</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
         <is>
-          <t>Obbligo di comunicazione dei dati relativi ai trasferimenti da e verso l'estero per intermediari finanziari e operatori.</t>
+          <t>Trasmettere all'Agenzia delle Entrate i dati sui trasferimenti transfrontalieri come banca o intermediario finanziario: obbligo per contrastare l'evasione tramite operazioni non canalizzate su conti italiani.</t>
         </is>
       </c>
     </row>
@@ -3858,7 +3958,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Fornire informazioni sulle operazioni con l'estero (monitoraggio fiscale)</t>
+          <t>Rispondere alle richieste di informazioni sui movimenti finanziari transfrontalieri</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3873,7 +3973,12 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Fornire informazioni sulle operazioni con l'estero (monitoraggio fiscale)</t>
+          <t>Rispondere alle richieste di informazioni sui movimenti finanziari transfrontalieri</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G76" t="inlineStr"/>
@@ -3900,12 +4005,12 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>Regular Business Operations — Gestione attività / Adempimenti ricorrenti</t>
+          <t>Regular Business Operations — Comunicazioni ricorrenti</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t>Richieste di informazioni sulle operazioni con l'estero nell'ambito del monitoraggio fiscale internazionale.</t>
+          <t>Rispondere alle richieste dell'Agenzia delle Entrate su movimenti finanziari transfrontalieri come intermediario: fornire dettagli su specifiche operazioni oggetto di indagine per controllo antievasione.</t>
         </is>
       </c>
     </row>
@@ -5159,7 +5264,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Dichiarazioni di intento</t>
+          <t>Presentare la dichiarazione d'intento come esportatore abituale</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -5170,13 +5275,38 @@
       <c r="D104" t="inlineStr">
         <is>
           <t>Dichiarazioni</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Presentare la dichiarazione d'intento come esportatore abituale</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="inlineStr"/>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Aprire e gestire un'attività o Partita IVA</t>
+        </is>
+      </c>
       <c r="K104" t="inlineStr">
         <is>
           <t>Guida IVA per imprese e professionisti</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti ricorrenti</t>
+        </is>
+      </c>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t>Presentare la dichiarazione d'intento come esportatore abituale: comunicare all'Agenzia delle Entrate l'intenzione di acquistare beni e servizi senza applicazione dell'IVA, entro il plafond disponibile.</t>
         </is>
       </c>
     </row>
@@ -5186,7 +5316,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Redditi società di capitali 2026</t>
+          <t>Presentare il Modello Redditi SC 2026 come società di capitali</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -5197,13 +5327,38 @@
       <c r="D105" t="inlineStr">
         <is>
           <t>Dichiarazioni</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Presentare il Modello Redditi SC 2026 come società di capitali</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="inlineStr"/>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Compilare ed inviare dichiarazioni</t>
+        </is>
+      </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>Dichiarazione dei redditi (730, Redditi PF)</t>
+          <t>Dichiarazioni imprese e societa'</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti annuali</t>
+        </is>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>Presentare il Modello Redditi Società di Capitali (SC) 2026 come SpA, Srl o cooperativa: dichiarare i redditi dell'anno d'imposta 2025 e liquidare IRES e IRAP entro le scadenze previste.</t>
         </is>
       </c>
     </row>
@@ -5213,7 +5368,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Certificazione unica 2026</t>
+          <t>Presentare la Certificazione Unica (CU) 2026 come sostituto d'imposta</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -5224,13 +5379,38 @@
       <c r="D106" t="inlineStr">
         <is>
           <t>Dichiarazioni</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Presentare la Certificazione Unica (CU) 2026 come sostituto d'imposta</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="inlineStr"/>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Compilare ed inviare dichiarazioni</t>
+        </is>
+      </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>Dichiarazioni sostituti d'imposta</t>
+          <t>Dichiarazioni imprese e societa'</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti annuali</t>
+        </is>
+      </c>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>Presentare la Certificazione Unica 2026 come sostituto d'imposta (datore di lavoro, ente pagante): attestare redditi corrisposti e ritenute operate su lavoratori dipendenti, autonomi e assimilati nel 2025.</t>
         </is>
       </c>
     </row>
@@ -5240,7 +5420,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Dichiarazioni per beneficiare della non imponibilità dell’Iva sui servizi di locazione, anche finanziaria, noleggio e simili, non a breve termine di imbarcazioni da diporto e di navigazione in alto mare</t>
+          <t>Presentare la dichiarazione della non imponibilità IVA (percentuali di detraibilità)</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -5251,10 +5431,40 @@
       <c r="D107" t="inlineStr">
         <is>
           <t>Dichiarazioni</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Presentare la dichiarazione della non imponibilità IVA (percentuali di detraibilità)</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr"/>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Aprire e gestire un'attività o Partita IVA</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>Guida IVA per imprese e professionisti</t>
+        </is>
+      </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti ricorrenti</t>
+        </is>
+      </c>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t>Presentare la dichiarazione delle percentuali di non imponibilità IVA come impresa mista: comunicare la percentuale di detraibilità applicabile in caso di operazioni sia imponibili sia esenti.</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -5262,7 +5472,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>770/2026</t>
+          <t>Presentare il Modello 770/2026 come sostituto d'imposta</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -5273,13 +5483,38 @@
       <c r="D108" t="inlineStr">
         <is>
           <t>Dichiarazioni</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Presentare il Modello 770/2026 come sostituto d'imposta</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G108" t="inlineStr"/>
       <c r="H108" t="inlineStr"/>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Compilare ed inviare dichiarazioni</t>
+        </is>
+      </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>Dichiarazioni sostituti d'imposta</t>
+          <t>Dichiarazioni imprese e societa'</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti annuali</t>
+        </is>
+      </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>Presentare il Modello 770/2026 come sostituto d'imposta: dichiarare le ritenute alla fonte operate nel 2025 su redditi da lavoro dipendente, autonomo e altri e le imposte sostitutive versate.</t>
         </is>
       </c>
     </row>
@@ -5351,7 +5586,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Dichiarazione d’imposta sostitutiva sui finanziamenti</t>
+          <t>Presentare la dichiarazione dell'imposta sostitutiva sui finanziamenti</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -5362,10 +5597,40 @@
       <c r="D110" t="inlineStr">
         <is>
           <t>Dichiarazioni</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Presentare la dichiarazione dell'imposta sostitutiva sui finanziamenti</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr"/>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>Compilare ed inviare dichiarazioni</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>Dichiarazioni imprese e societa'</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti annuali</t>
+        </is>
+      </c>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t>Presentare la dichiarazione dell'imposta sostitutiva sui finanziamenti come banca o intermediario: dichiarare i finanziamenti a medio-lungo termine assoggettati all'imposta sostitutiva dello 0,25%.</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -5373,7 +5638,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Iva base 2026</t>
+          <t>Presentare la dichiarazione IVA Base 2026 come piccolo contribuente</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -5384,13 +5649,38 @@
       <c r="D111" t="inlineStr">
         <is>
           <t>Dichiarazioni</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Presentare la dichiarazione IVA Base 2026 come piccolo contribuente</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr"/>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Compilare ed inviare dichiarazioni</t>
+        </is>
+      </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>Guida IVA per imprese e professionisti</t>
+          <t>Dichiarazioni imprese e societa'</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti annuali</t>
+        </is>
+      </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>Presentare la dichiarazione IVA Base 2026 come piccolo contribuente: versione semplificata della dichiarazione annuale IVA, per soggetti con operazioni semplici e senza regimi particolari.</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5690,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Redditi Enti non commerciali Enc 2026</t>
+          <t>Presentare il Modello Redditi ENC 2026 come ente non commerciale</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -5411,13 +5701,38 @@
       <c r="D112" t="inlineStr">
         <is>
           <t>Dichiarazioni</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Presentare il Modello Redditi ENC 2026 come ente non commerciale</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G112" t="inlineStr"/>
       <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>Compilare ed inviare dichiarazioni</t>
+        </is>
+      </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>Dichiarazione dei redditi (730, Redditi PF)</t>
+          <t>Dichiarazioni imprese e societa'</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti annuali</t>
+        </is>
+      </c>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>Presentare il Modello Redditi Enti Non Commerciali (ENC) 2026 come ente non commerciale, associazione, fondazione o ONLUS: dichiarare redditi commerciali e non commerciali dell'anno 2025.</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5742,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Dichiarazione precompilata</t>
+          <t>Consultare e inviare la dichiarazione precompilata come cittadino</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -5438,13 +5753,38 @@
       <c r="D113" t="inlineStr">
         <is>
           <t>Dichiarazioni</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Consultare e inviare la dichiarazione precompilata come cittadino</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G113" t="inlineStr"/>
       <c r="H113" t="inlineStr"/>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>Compilare ed inviare dichiarazioni</t>
+        </is>
+      </c>
       <c r="K113" t="inlineStr">
         <is>
           <t>Dichiarazione dei redditi (730, Redditi PF)</t>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>Life events — Dichiarazione dei redditi</t>
+        </is>
+      </c>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>Consultare e inviare la dichiarazione dei redditi precompilata come cittadino: accedere al modello 730 o Redditi PF già precaricato con i dati di redditi, oneri detraibili e ritenute.</t>
         </is>
       </c>
     </row>
@@ -5454,7 +5794,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Cupe</t>
+          <t>Presentare la Certificazione degli utili (CUPE) come società erogante</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -5465,13 +5805,38 @@
       <c r="D114" t="inlineStr">
         <is>
           <t>Dichiarazioni</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Presentare la Certificazione degli utili (CUPE) come società erogante</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="inlineStr"/>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Compilare ed inviare dichiarazioni</t>
+        </is>
+      </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>Dichiarazioni sostituti d'imposta</t>
+          <t>Dichiarazioni imprese e societa'</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti annuali</t>
+        </is>
+      </c>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>Presentare la Certificazione degli Utili (CUPE) come società di capitali erogante: attestare i dividendi e gli utili corrisposti ai soci nel 2025 con le relative ritenute d'acconto applicate.</t>
         </is>
       </c>
     </row>
@@ -5481,7 +5846,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>770/2026</t>
+          <t>Presentare il Modello 770/2026 come sostituto d'imposta (variante)</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -5492,13 +5857,38 @@
       <c r="D115" t="inlineStr">
         <is>
           <t>Dichiarazioni</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Presentare il Modello 770/2026 come sostituto d'imposta (variante)</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr"/>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Compilare ed inviare dichiarazioni</t>
+        </is>
+      </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>Dichiarazioni sostituti d'imposta</t>
+          <t>Dichiarazioni imprese e societa'</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti annuali</t>
+        </is>
+      </c>
+      <c r="N115" t="inlineStr">
+        <is>
+          <t>DUPLICATO di ID 173 — da verificare accorpamento. Scheda 770/2026 per sostituto d'imposta: dichiarazione delle ritenute alla fonte operate nel 2025.</t>
         </is>
       </c>
     </row>
@@ -5508,7 +5898,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Iva 2026</t>
+          <t>Presentare la dichiarazione IVA 2026 come impresa</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -5519,13 +5909,38 @@
       <c r="D116" t="inlineStr">
         <is>
           <t>Dichiarazioni</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Presentare la dichiarazione IVA 2026 come impresa</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G116" t="inlineStr"/>
       <c r="H116" t="inlineStr"/>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Compilare ed inviare dichiarazioni</t>
+        </is>
+      </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>Guida IVA per imprese e professionisti</t>
+          <t>Dichiarazioni imprese e societa'</t>
+        </is>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti annuali</t>
+        </is>
+      </c>
+      <c r="N116" t="inlineStr">
+        <is>
+          <t>Presentare la dichiarazione annuale IVA 2026 come impresa o professionista: liquidare l'IVA dovuta o a credito per l'anno d'imposta 2025 e chiudere gli obblighi periodici IVA.</t>
         </is>
       </c>
     </row>
@@ -5535,7 +5950,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Redditi società di persone 2026</t>
+          <t>Presentare il Modello Redditi SP 2026 come società di persone</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -5546,13 +5961,38 @@
       <c r="D117" t="inlineStr">
         <is>
           <t>Dichiarazioni</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Presentare il Modello Redditi SP 2026 come società di persone</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr"/>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Compilare ed inviare dichiarazioni</t>
+        </is>
+      </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>Dichiarazione dei redditi (730, Redditi PF)</t>
+          <t>Dichiarazioni imprese e societa'</t>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti annuali</t>
+        </is>
+      </c>
+      <c r="N117" t="inlineStr">
+        <is>
+          <t>Presentare il Modello Redditi Società di Persone (SP) 2026 come Snc, Sas o studio associato: dichiarare i redditi del 2025 attribuiti pro-quota ai soci.</t>
         </is>
       </c>
     </row>
@@ -7446,7 +7886,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Registrare online un atto o un contratto firmato digitalmente</t>
+          <t>Registrare un atto firmato digitalmente</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -7461,7 +7901,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Registrare online un atto o un contratto firmato digitalmente</t>
+          <t>Registrare un atto firmato digitalmente</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
@@ -7473,7 +7913,7 @@
       <c r="H155" t="inlineStr"/>
       <c r="I155" t="inlineStr">
         <is>
-          <t>Certificati e attestazioni</t>
+          <t>Richieste e comunicazioni all'Agenzia</t>
         </is>
       </c>
       <c r="K155" t="inlineStr">
@@ -7483,12 +7923,12 @@
       </c>
       <c r="M155" t="inlineStr">
         <is>
-          <t>Regular Business Operations — Gestione attività / Adempimenti ricorrenti</t>
+          <t>Regular Business Operations — Adempimenti ricorrenti</t>
         </is>
       </c>
       <c r="N155" t="inlineStr">
         <is>
-          <t>Procedura per la registrazione telematica degli atti con firma digitale.</t>
+          <t>Registrare un atto firmato digitalmente come parte contraente o professionista: presentare l'atto in formato elettronico all'ufficio dell'Agenzia delle Entrate senza necessità di copia cartacea.</t>
         </is>
       </c>
     </row>
@@ -7550,7 +7990,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Certificato sull'esistenza di contestazioni in corso e di quelle già definite per le quali i debiti non sono stati soddisfatti” (art. 14 del D.Lgs. 18 dicembre 1997, n. 472).</t>
+          <t>Richiedere il certificato sull'esistenza di contestazioni fiscali in corso</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -7561,10 +8001,40 @@
       <c r="D157" t="inlineStr">
         <is>
           <t>Istanze</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Richiedere il certificato sull'esistenza di contestazioni fiscali in corso</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G157" t="inlineStr"/>
       <c r="H157" t="inlineStr"/>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>Certificati e attestazioni</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>Certificati fiscali</t>
+        </is>
+      </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti ricorrenti</t>
+        </is>
+      </c>
+      <c r="N157" t="inlineStr">
+        <is>
+          <t>Richiedere il certificato sull'esistenza di contestazioni fiscali in corso come contribuente o interessato: attestazione ufficiale della presenza di procedimenti pendenti presso l'Agenzia delle Entrate.</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -7738,7 +8208,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Deleghe servizi online Agenzia delle Entrate - Riscossione</t>
+          <t>Delegare l'accesso ai servizi online di Agenzia delle Entrate-Riscossione</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -7749,10 +8219,40 @@
       <c r="D161" t="inlineStr">
         <is>
           <t>Istanze</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Delegare l'accesso ai servizi online di Agenzia delle Entrate-Riscossione</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>Scheda istanza</t>
         </is>
       </c>
       <c r="G161" t="inlineStr"/>
       <c r="H161" t="inlineStr"/>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>Richieste e comunicazioni all'Agenzia</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>Deleghe e abilitazioni</t>
+        </is>
+      </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>Life events — Amministrazione fiscale</t>
+        </is>
+      </c>
+      <c r="N161" t="inlineStr">
+        <is>
+          <t>Delegare un intermediario o familiare per accedere ai servizi online dell'Agenzia delle Entrate-Riscossione come contribuente: autorizzare la consultazione della propria posizione debitoria e la gestione di rateizzazioni.</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -7760,7 +8260,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Identificazione Iva soggetti non residenti (Anr/3)</t>
+          <t>Registrarsi ai fini IVA come soggetto non residente (Modello ANR/3)</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -7771,6 +8271,11 @@
       <c r="D162" t="inlineStr">
         <is>
           <t>Istanze</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>Registrarsi ai fini IVA come soggetto non residente (Modello ANR/3)</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
@@ -7792,12 +8297,12 @@
       </c>
       <c r="M162" t="inlineStr">
         <is>
-          <t>Business Start-Up — Avvio attività / Apertura P.IVA</t>
+          <t>Regular Business Operations — Attività internazionale</t>
         </is>
       </c>
       <c r="N162" t="inlineStr">
         <is>
-          <t>Procedura per l'identificazione ai fini IVA di soggetti non residenti mediante il modello ANR/3, per svolgere attività imponibili in Italia.</t>
+          <t>Registrarsi ai fini IVA come soggetto non residente tramite identificazione diretta (Modello ANR/3): ottenere una posizione IVA italiana senza rappresentante fiscale, per operatori UE.</t>
         </is>
       </c>
     </row>
@@ -8124,7 +8629,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Richiedere il certificato unico dei debiti tributari</t>
+          <t>Richiedere il certificato unico dei debiti tributari (CUDT)</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -8139,7 +8644,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Richiedere il certificato unico dei debiti tributari</t>
+          <t>Richiedere il certificato unico dei debiti tributari (CUDT)</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
@@ -8161,12 +8666,12 @@
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>Starting a Small Claims Procedure — Contenzioso fiscale / Procedure legali</t>
+          <t>Regular Business Operations — Adempimenti straordinari</t>
         </is>
       </c>
       <c r="N169" t="inlineStr">
         <is>
-          <t>Richiesta del certificato unico dei debiti tributari, che attesta i debiti risultanti a carico del contribuente.</t>
+          <t>Richiedere il Certificato Unico dei Debiti Tributari (CUDT) come contribuente o curatore: attestazione dei debiti tributari accertati e non pagati verso l'Agenzia delle Entrate.</t>
         </is>
       </c>
     </row>
@@ -8815,7 +9320,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Richiedere il certificato di regolarità fiscale (Carichi pendenti)</t>
+          <t>Richiedere il certificato dei carichi pendenti fiscali</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -8830,7 +9335,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>Richiedere il certificato di regolarità fiscale (Carichi pendenti)</t>
+          <t>Richiedere il certificato dei carichi pendenti fiscali</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
@@ -8852,12 +9357,12 @@
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>Starting a Small Claims Procedure — Contenzioso fiscale / Procedure legali</t>
+          <t>Regular Business Operations — Adempimenti straordinari</t>
         </is>
       </c>
       <c r="N182" t="inlineStr">
         <is>
-          <t>Certificato dei carichi pendenti: attesta l'esistenza di contestazioni in corso e di quelle definite a carico del contribuente.</t>
+          <t>Richiedere il certificato dei carichi pendenti come contribuente: attestazione ufficiale delle contestazioni fiscali pendenti utile per compravendite d'azienda, gare pubbliche o operazioni straordinarie.</t>
         </is>
       </c>
     </row>
@@ -10445,7 +10950,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Imposta di registro</t>
+          <t>Pagare l'imposta di registro sui contratti</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -10456,6 +10961,11 @@
       <c r="D212" t="inlineStr">
         <is>
           <t>Pagamenti</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Pagare l'imposta di registro sui contratti</t>
         </is>
       </c>
       <c r="F212" t="inlineStr">
@@ -10465,6 +10975,26 @@
       </c>
       <c r="G212" t="inlineStr"/>
       <c r="H212" t="inlineStr"/>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>Pagamenti e Rimborsi</t>
+        </is>
+      </c>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>Istruzioni per il pagamento delle imposte</t>
+        </is>
+      </c>
+      <c r="M212" t="inlineStr">
+        <is>
+          <t>Property purchase / renovation — Contratti</t>
+        </is>
+      </c>
+      <c r="N212" t="inlineStr">
+        <is>
+          <t>Pagare l'imposta di registro sui contratti come parte contraente: versare l'imposta dovuta per la registrazione di contratti di locazione, compravendita, comodato o altri atti soggetti a registrazione.</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -11627,2362 +12157,2897 @@
     </row>
     <row r="235">
       <c r="A235" t="n">
-        <v>462</v>
+        <v>384</v>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Ravvedimento Cpb annualità 2019-2023</t>
+          <t>Pagamenti</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/ravvedimento-cpb-annualita-2019-2023</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Pagamenti/</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>Accertamenti e regolarizzazioni</t>
+          <t>ADER - Pagamenti</t>
         </is>
       </c>
       <c r="G235" t="inlineStr"/>
       <c r="H235" t="inlineStr"/>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>Pagamenti e Rimborsi</t>
+        </is>
+      </c>
+      <c r="K235" t="inlineStr">
+        <is>
+          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="n">
-        <v>464</v>
+        <v>385</v>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Ravvedimento Cpb annualità 2018-2022</t>
+          <t>Come e dove pagare</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/ravvedimento-cpb</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Pagamenti/comedovepagare/</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>Accertamenti e regolarizzazioni</t>
+          <t>ADER - Pagamenti - Come e dove pagare</t>
         </is>
       </c>
       <c r="G236" t="inlineStr"/>
       <c r="H236" t="inlineStr"/>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>Pagamenti e Rimborsi</t>
+        </is>
+      </c>
+      <c r="K236" t="inlineStr">
+        <is>
+          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="n">
-        <v>466</v>
+        <v>386</v>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Richiedere il credito d'imposta aggiuntivo per investimenti nella ZES unica 2025</t>
+          <t>Pagamenti dall'estero</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/credito-d-imposta-aggiuntivo-zes-unica-2025</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Pagamenti/PagamentiDallEstero/</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>Agevolazioni</t>
-        </is>
-      </c>
-      <c r="E237" t="inlineStr">
-        <is>
-          <t>Richiedere il credito d'imposta aggiuntivo per investimenti nella ZES unica 2025</t>
+          <t>ADER - Pagamenti - Pagamenti dall'estero</t>
         </is>
       </c>
       <c r="G237" t="inlineStr"/>
       <c r="H237" t="inlineStr"/>
       <c r="I237" t="inlineStr">
         <is>
-          <t>Ottenere bonus e agevolazioni</t>
+          <t>Pagamenti e Rimborsi</t>
+        </is>
+      </c>
+      <c r="J237" t="inlineStr">
+        <is>
+          <t>Fiscalità internazionale e residenti all'estero</t>
         </is>
       </c>
       <c r="K237" t="inlineStr">
         <is>
-          <t>Agevolazioni imprese e start-up</t>
+          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
+        </is>
+      </c>
+      <c r="M237" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Gestione attività / Adempimenti ricorrenti</t>
+        </is>
+      </c>
+      <c r="N237" t="inlineStr">
+        <is>
+          <t>Servizio per cittadini residenti all'estero per pagare cartelle e avvisi tramite pagoPA, bonifico bancario o canali telematici.</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="n">
-        <v>467</v>
+        <v>387</v>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>Richiedere il credito d'imposta per cuochi professionisti</t>
+          <t>Compensazioni</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/credito-di-imposta-per-cuochi-professionisti</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Compensazioni/</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>Agevolazioni</t>
-        </is>
-      </c>
-      <c r="E238" t="inlineStr">
-        <is>
-          <t>Richiedere il credito d'imposta per cuochi professionisti</t>
+          <t>ADER - Compensazioni</t>
         </is>
       </c>
       <c r="G238" t="inlineStr"/>
       <c r="H238" t="inlineStr"/>
       <c r="I238" t="inlineStr">
         <is>
-          <t>Ottenere bonus e agevolazioni</t>
+          <t>Pagamenti e Rimborsi</t>
         </is>
       </c>
       <c r="K238" t="inlineStr">
         <is>
-          <t>Agevolazioni imprese e start-up</t>
-        </is>
-      </c>
-      <c r="N238" t="inlineStr">
-        <is>
-          <t>Richiedere il credito d'imposta per cuochi professionisti come lavoratore autonomo o dipendente del settore: agevolazione su acquisto strumenti professionali, fruibile tramite F24 in compensazione.</t>
+          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="n">
-        <v>468</v>
+        <v>388</v>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Richiedere il contributo a fondo perduto per interventi edilizi 2024</t>
+          <t>Rateizzazione</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/contributo-a-fondo-perduto-per-interventi-edilizi-2024</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rateizzazione/</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>Agevolazioni</t>
-        </is>
-      </c>
-      <c r="E239" t="inlineStr">
-        <is>
-          <t>Richiedere il contributo a fondo perduto per interventi edilizi 2024</t>
+          <t>ADER - Rateizzazione</t>
         </is>
       </c>
       <c r="G239" t="inlineStr"/>
       <c r="H239" t="inlineStr"/>
       <c r="I239" t="inlineStr">
         <is>
-          <t>Ottenere bonus e agevolazioni</t>
+          <t>Pagamenti e Rimborsi</t>
         </is>
       </c>
       <c r="K239" t="inlineStr">
         <is>
-          <t>Agevolazioni casa e ristrutturazioni</t>
+          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="n">
-        <v>469</v>
+        <v>389</v>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Ottenere le agevolazioni per il primo insediamento di imprese giovanili in agricoltura</t>
+          <t xml:space="preserve"> La  rateizzazione dal 1° gennaio 2025</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/primo-insediamento-delle-imprese-giovanili-in-agricoltura</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rateizzazione/la-rateizzazione/</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>Agevolazioni</t>
-        </is>
-      </c>
-      <c r="E240" t="inlineStr">
-        <is>
-          <t>Ottenere le agevolazioni per il primo insediamento di imprese giovanili in agricoltura</t>
+          <t>ADER - Rateizzazione - La rateizzazione dal 1° gennaio 2025</t>
         </is>
       </c>
       <c r="G240" t="inlineStr"/>
       <c r="H240" t="inlineStr"/>
       <c r="I240" t="inlineStr">
         <is>
-          <t>Ottenere bonus e agevolazioni</t>
-        </is>
-      </c>
-      <c r="J240" t="inlineStr">
-        <is>
-          <t>Aprire e gestire un'attività o Partita IVA</t>
+          <t>Pagamenti e Rimborsi</t>
         </is>
       </c>
       <c r="K240" t="inlineStr">
         <is>
-          <t>Agevolazioni imprese e start-up</t>
-        </is>
-      </c>
-      <c r="L240" t="inlineStr">
-        <is>
-          <t>Avviare un'attività</t>
-        </is>
-      </c>
-      <c r="N240" t="inlineStr">
-        <is>
-          <t>Ottenere le agevolazioni per il primo insediamento di imprenditori agricoli come giovane sotto i 41 anni: contributi e benefici fiscali sul reddito d'impresa per chi avvia un'attività agricola.</t>
+          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="n">
-        <v>470</v>
+        <v>390</v>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>Richiedere il credito d'imposta per la formazione in gestione agricola</t>
+          <t>Istanze "a semplice richiesta"</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/credito-d-imposta-per-le-spese-sostenute-per-la-partecipazione-a-corsi-di-formazione-attinenti-alla-gestione-dell-azienda-agricola</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rateizzazione/istanze-a-semplice-richiesta/</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>Agevolazioni</t>
-        </is>
-      </c>
-      <c r="E241" t="inlineStr">
-        <is>
-          <t>Richiedere il credito d'imposta per la formazione in gestione agricola</t>
+          <t>ADER - Rateizzazione - Istanze "a semplice richiesta"</t>
         </is>
       </c>
       <c r="G241" t="inlineStr"/>
       <c r="H241" t="inlineStr"/>
       <c r="I241" t="inlineStr">
         <is>
-          <t>Ottenere bonus e agevolazioni</t>
+          <t>Pagamenti e Rimborsi</t>
         </is>
       </c>
       <c r="K241" t="inlineStr">
         <is>
-          <t>Agevolazioni imprese e start-up</t>
-        </is>
-      </c>
-      <c r="N241" t="inlineStr">
-        <is>
-          <t>Richiedere il credito d'imposta per la formazione in gestione d'impresa come imprenditore: agevolazione su corsi di alta formazione manageriale, fruibile in compensazione tramite F24.</t>
+          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="n">
-        <v>472</v>
+        <v>391</v>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Iscriversi al contributo del 5 per mille</t>
+          <t>Istanze "documentate"</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/contributo-del-5-per-mille-anno-2026</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rateizzazione/istanze-documentate/</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>Agevolazioni</t>
-        </is>
-      </c>
-      <c r="E242" t="inlineStr">
-        <is>
-          <t>Iscriversi al contributo del 5 per mille</t>
-        </is>
-      </c>
-      <c r="F242" t="inlineStr">
-        <is>
-          <t>Scheda complessa</t>
+          <t>ADER - Rateizzazione - Istanze "documentate"</t>
         </is>
       </c>
       <c r="G242" t="inlineStr"/>
       <c r="H242" t="inlineStr"/>
       <c r="I242" t="inlineStr">
         <is>
-          <t>Ottenere bonus e agevolazioni</t>
+          <t>Pagamenti e Rimborsi</t>
         </is>
       </c>
       <c r="K242" t="inlineStr">
         <is>
-          <t>Enti del Terzo Settore</t>
-        </is>
-      </c>
-      <c r="N242" t="inlineStr">
-        <is>
-          <t>Iscriversi al contributo del 5 per mille come ente del Terzo Settore, ONLUS, associazione, ente di ricerca o altro soggetto ammesso: presentazione domanda e mantenimento dei requisiti per ricevere le quote IRPEF dei contribuenti.</t>
+          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="n">
-        <v>474</v>
+        <v>392</v>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Aderire al regime IVA transfrontaliero di franchigia</t>
+          <t>Proroga del piano di rateizzazione</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/nuovo-regime-iva-per-le-piccole-imprese</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rateizzazione/Proroga/</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>Agevolazioni</t>
-        </is>
-      </c>
-      <c r="E243" t="inlineStr">
-        <is>
-          <t>Aderire al regime IVA transfrontaliero di franchigia</t>
+          <t>ADER - Rateizzazione - Proroga del piano di rateizzazione</t>
         </is>
       </c>
       <c r="G243" t="inlineStr"/>
       <c r="H243" t="inlineStr"/>
       <c r="I243" t="inlineStr">
         <is>
-          <t>Ottenere bonus e agevolazioni</t>
-        </is>
-      </c>
-      <c r="J243" t="inlineStr">
-        <is>
-          <t>Fiscalità internazionale e residenti all'estero</t>
+          <t>Pagamenti e Rimborsi</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
         <is>
-          <t>Regimi opzionali per le imprese e professionisti</t>
-        </is>
-      </c>
-      <c r="L243" t="inlineStr">
-        <is>
-          <t>IVA e adempimenti</t>
-        </is>
-      </c>
-      <c r="N243" t="inlineStr">
-        <is>
-          <t>Aderire al regime IVA transfrontaliero di franchigia come piccola impresa: regime che esonera dall'addebito IVA negli altri Stati UE in cui si vendono beni o servizi, soglia di volume d'affari 100.000€ annui.</t>
+          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="n">
-        <v>475</v>
+        <v>393</v>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>Adottare il sistema di controllo del rischio fiscale</t>
+          <t>Istanze "documentate" - Indicatori</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/regime-opzionale-di-adozione-del-sistema-di-controllo-del-rischio-fiscale</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rateizzazione/istanze-documentate-indicatori/</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>Agevolazioni</t>
-        </is>
-      </c>
-      <c r="E244" t="inlineStr">
-        <is>
-          <t>Adottare il sistema di controllo del rischio fiscale</t>
+          <t>ADER - Rateizzazione - Istanze "documentate" - Indicatori</t>
         </is>
       </c>
       <c r="G244" t="inlineStr"/>
       <c r="H244" t="inlineStr"/>
       <c r="I244" t="inlineStr">
         <is>
-          <t>Ottenere bonus e agevolazioni</t>
+          <t>Pagamenti e Rimborsi</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
         <is>
-          <t>Regimi opzionali per le imprese e professionisti</t>
-        </is>
-      </c>
-      <c r="N244" t="inlineStr">
-        <is>
-          <t>Adottare il sistema di controllo del rischio fiscale (Tax Control Framework, TCF) come grande impresa: insieme di procedure interne per identificare, misurare e gestire il rischio fiscale, requisito per la cooperative compliance.</t>
+          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="n">
-        <v>476</v>
+        <v>394</v>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>Richiedere il credito d'imposta per investimenti nella ZES unica 2026</t>
+          <t>Istanze "documentate" - Simula il numero delle rate</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/credito-d-imposta-per-investimenti-nella-zes-unica-zes-2026-</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rateizzazione/istanze-documentate-simula-il-numero-delle-rate/</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>Agevolazioni</t>
-        </is>
-      </c>
-      <c r="E245" t="inlineStr">
-        <is>
-          <t>Richiedere il credito d'imposta per investimenti nella ZES unica 2026</t>
+          <t>ADER - Rateizzazione - Istanze "documentate" - Simula il numero delle rate</t>
         </is>
       </c>
       <c r="G245" t="inlineStr"/>
       <c r="H245" t="inlineStr"/>
       <c r="I245" t="inlineStr">
         <is>
-          <t>Ottenere bonus e agevolazioni</t>
+          <t>Pagamenti e Rimborsi</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
         <is>
-          <t>Agevolazioni imprese e start-up</t>
-        </is>
-      </c>
-      <c r="N245" t="inlineStr">
-        <is>
-          <t>Richiedere il credito d'imposta per investimenti nella ZES (Zona Economica Speciale) unica del Mezzogiorno come impresa (annualità 2026): agevolazione su beni strumentali nuovi, fruibile in compensazione tramite F24.</t>
+          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="n">
-        <v>477</v>
+        <v>395</v>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>Richiedere il credito d'imposta per investimenti nelle ZLS 2026</t>
+          <t>Cosa succede con la presentazione della richiesta di rateizzazione</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/zls-2026</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rateizzazione/cosa-succede-con-la-presentazione-della-richiesta-di-rateizzazione/</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>Agevolazioni</t>
-        </is>
-      </c>
-      <c r="E246" t="inlineStr">
-        <is>
-          <t>Richiedere il credito d'imposta per investimenti nelle ZLS 2026</t>
+          <t>ADER - Rateizzazione - Cosa succede con la presentazione della richiesta</t>
         </is>
       </c>
       <c r="G246" t="inlineStr"/>
       <c r="H246" t="inlineStr"/>
       <c r="I246" t="inlineStr">
         <is>
-          <t>Ottenere bonus e agevolazioni</t>
+          <t>Pagamenti e Rimborsi</t>
         </is>
       </c>
       <c r="K246" t="inlineStr">
         <is>
-          <t>Agevolazioni imprese e start-up</t>
-        </is>
-      </c>
-      <c r="N246" t="inlineStr">
-        <is>
-          <t>Richiedere il credito d'imposta per investimenti nelle aree del Centro Italia colpite dal sisma come impresa: agevolazione fiscale per ripresa economica, fruibile in compensazione tramite F24.</t>
+          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="n">
-        <v>478</v>
+        <v>396</v>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>Comunicare il regime IVA transfrontaliero di franchigia</t>
+          <t>Decadenza dal piano di rateizzazione</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/comunicazione-trimestrale-del-regime-transfrontaliero-di-franchigia</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rateizzazione/decadenza-dal-piano-di-rateizzazione/</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>Comunicazioni</t>
-        </is>
-      </c>
-      <c r="E247" t="inlineStr">
-        <is>
-          <t>Comunicare il regime IVA transfrontaliero di franchigia</t>
+          <t>ADER - Rateizzazione - Decadenza dal piano di rateizzazione</t>
         </is>
       </c>
       <c r="G247" t="inlineStr"/>
       <c r="H247" t="inlineStr"/>
       <c r="I247" t="inlineStr">
         <is>
-          <t>Aprire e gestire un'attività o Partita IVA</t>
-        </is>
-      </c>
-      <c r="J247" t="inlineStr">
-        <is>
-          <t>Fiscalità internazionale e residenti all'estero</t>
+          <t>Pagamenti e Rimborsi</t>
         </is>
       </c>
       <c r="K247" t="inlineStr">
         <is>
-          <t>Guida IVA per imprese e professionisti</t>
-        </is>
-      </c>
-      <c r="L247" t="inlineStr">
-        <is>
-          <t>IVA e adempimenti</t>
-        </is>
-      </c>
-      <c r="N247" t="inlineStr">
-        <is>
-          <t>Comunicare l'adesione al regime IVA transfrontaliero di franchigia come piccola impresa: adempimento obbligatorio per beneficiare dell'esonero IVA negli altri Stati UE, con monitoraggio della soglia 100.000€.</t>
+          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="n">
-        <v>479</v>
+        <v>397</v>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>Optare per il regime IVA per servizi di trasporto e logistica</t>
+          <t>Rateizzazione - Domiciliazione bancaria</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/opzione-per-le-prestazioni-di-servizi-rese-nei-confronti-di-imprese-che-svolgono-attivita-di-trasporto-movimentazione-merci-e-servizi-di-logistica</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rateizzazione/rateizzazione-domiciliazione-bancaria/</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>Comunicazioni</t>
-        </is>
-      </c>
-      <c r="E248" t="inlineStr">
-        <is>
-          <t>Optare per il regime IVA per servizi di trasporto e logistica</t>
+          <t>ADER - Rateizzazione - Domiciliazione bancaria</t>
         </is>
       </c>
       <c r="G248" t="inlineStr"/>
       <c r="H248" t="inlineStr"/>
       <c r="I248" t="inlineStr">
         <is>
-          <t>Aprire e gestire un'attività o Partita IVA</t>
+          <t>Pagamenti e Rimborsi</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
         <is>
-          <t>Guida IVA per imprese e professionisti</t>
-        </is>
-      </c>
-      <c r="N248" t="inlineStr">
-        <is>
-          <t>Optare per il regime IVA dedicato ai servizi di trasporto e logistica internazionale come impresa del settore: regole specifiche su esenzioni e applicazione dell'IVA nei trasporti intra-UE ed extra-UE.</t>
+          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="n">
-        <v>480</v>
+        <v>398</v>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>Comunicare le spese sanitarie sostenute</t>
+          <t>Rateizzazione - Richiedi i moduli di pagamento</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/spese-sanitarie</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rateizzazione/bollettini-moduli-di-pagamento/</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>Comunicazioni</t>
-        </is>
-      </c>
-      <c r="E249" t="inlineStr">
-        <is>
-          <t>Comunicare le spese sanitarie sostenute</t>
+          <t>ADER - Rateizzazione - Richiedi i moduli di pagamento</t>
         </is>
       </c>
       <c r="G249" t="inlineStr"/>
       <c r="H249" t="inlineStr"/>
       <c r="I249" t="inlineStr">
         <is>
-          <t>Compilare ed inviare dichiarazioni</t>
+          <t>Pagamenti e Rimborsi</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
         <is>
-          <t>Dati per la dichiarazione precompilata</t>
-        </is>
-      </c>
-      <c r="N249" t="inlineStr">
-        <is>
-          <t>Comunicare le spese sanitarie sostenute dai cittadini come struttura sanitaria, farmacia, medico o altro operatore: trasmissione al Sistema TS (Tessera Sanitaria) per la dichiarazione precompilata e la detrazione IRPEF.</t>
+          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="n">
-        <v>481</v>
+        <v>399</v>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Comunicare i proventi dalla cessione di energia da fonti rinnovabili</t>
+          <t>Enti che rateizzano in proprio e tributi/tipi imposta non rateizzabili</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/com_impianto_alimentato_fonti_derivabili</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rateizzazione/EntiCheRateizzanoInProprioETributiNonRateizzabili/</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>Comunicazioni</t>
-        </is>
-      </c>
-      <c r="E250" t="inlineStr">
-        <is>
-          <t>Comunicare i proventi dalla cessione di energia da fonti rinnovabili</t>
+          <t>ADER - Rateizzazione - Enti che rateizzano in proprio</t>
         </is>
       </c>
       <c r="G250" t="inlineStr"/>
       <c r="H250" t="inlineStr"/>
       <c r="I250" t="inlineStr">
         <is>
-          <t>Compilare ed inviare dichiarazioni</t>
+          <t>Pagamenti e Rimborsi</t>
         </is>
       </c>
       <c r="K250" t="inlineStr">
         <is>
-          <t>Dati per la dichiarazione precompilata</t>
-        </is>
-      </c>
-      <c r="N250" t="inlineStr">
-        <is>
-          <t>Comunicare i proventi dalla cessione di energia da fonti rinnovabili come gestore di impianto fotovoltaico, eolico o biomasse: trasmissione annuale al GSE e all'Agenzia ai fini fiscali.</t>
+          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="n">
-        <v>482</v>
+        <v>400</v>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Indicare il domicilio digitale (PEC) per ricevere atti e comunicazioni</t>
+          <t>Enti che hanno autorizzato l’Agente della riscossione a concedere la rateizzazione</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/comunicazione-del-domicilio-digitale-speciale</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rateizzazione/Enti-Rateizzazione/</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>Comunicazioni</t>
-        </is>
-      </c>
-      <c r="E251" t="inlineStr">
-        <is>
-          <t>Indicare il domicilio digitale (PEC) per ricevere atti e comunicazioni</t>
+          <t>ADER - Rateizzazione - Enti autorizzati alla riscossione</t>
         </is>
       </c>
       <c r="G251" t="inlineStr"/>
       <c r="H251" t="inlineStr"/>
       <c r="I251" t="inlineStr">
         <is>
-          <t>Richieste e comunicazioni all'Agenzia</t>
+          <t>Pagamenti e Rimborsi</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
         <is>
-          <t>Notifiche e domicilio digitale</t>
-        </is>
-      </c>
-      <c r="N251" t="inlineStr">
-        <is>
-          <t>Indicare il domicilio digitale (PEC, Posta Elettronica Certificata) per ricevere atti dall'Agenzia delle Entrate: comunicazione che permette notifica telematica di accertamenti, comunicazioni e provvedimenti.</t>
+          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="n">
-        <v>483</v>
+        <v>401</v>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>Delegare l'accesso ai servizi online dell'Agenzia delle Entrate e della Riscossione</t>
+          <t>Sospensione</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/delega-unica-ai-servizi-on-line-dell-agenzia-delle-entrate-e-dell-agenzia-delle-entrate-riscossione</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Sospensione/</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>Comunicazioni</t>
-        </is>
-      </c>
-      <c r="E252" t="inlineStr">
-        <is>
-          <t>Delegare l'accesso ai servizi online dell'Agenzia delle Entrate e della Riscossione</t>
+          <t>ADER - Sospensione</t>
         </is>
       </c>
       <c r="G252" t="inlineStr"/>
       <c r="H252" t="inlineStr"/>
       <c r="I252" t="inlineStr">
         <is>
-          <t>Richieste e comunicazioni all'Agenzia</t>
+          <t>Pagamenti e Rimborsi</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">
         <is>
-          <t>Deleghe e abilitazioni</t>
-        </is>
-      </c>
-      <c r="N252" t="inlineStr">
-        <is>
-          <t>Delegare l'accesso ai servizi online dell'Agenzia delle Entrate a un familiare, professionista o intermediario: procedura per autorizzare un terzo a operare sul proprio cassetto fiscale e dichiarazioni.</t>
+          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="n">
-        <v>484</v>
+        <v>402</v>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>Comunicare la cessazione dell'incarico di depositario delle scritture contabili</t>
+          <t>Annullamento del debito</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/comunicazione-di-cessazione-incarico-di-depositario-scritture-contabili</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/AnnullamentoDelDebito/</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>Comunicazioni</t>
-        </is>
-      </c>
-      <c r="E253" t="inlineStr">
-        <is>
-          <t>Comunicare la cessazione dell'incarico di depositario delle scritture contabili</t>
+          <t>ADER - Annullamento del debito</t>
         </is>
       </c>
       <c r="G253" t="inlineStr"/>
       <c r="H253" t="inlineStr"/>
       <c r="I253" t="inlineStr">
         <is>
-          <t>Aprire e gestire un'attività o Partita IVA</t>
+          <t>Pagamenti e Rimborsi</t>
         </is>
       </c>
       <c r="K253" t="inlineStr">
         <is>
-          <t>Avviare un'attività</t>
-        </is>
-      </c>
-      <c r="N253" t="inlineStr">
-        <is>
-          <t>Comunicare la cessazione dell'incarico come depositario delle scritture contabili: adempimento obbligatorio entro 30 giorni dalla rinuncia o revoca, comunicazione tramite modello AA9/12.</t>
+          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="n">
-        <v>485</v>
+        <v>403</v>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>Comunicare le transazioni con pagamenti elettronici</t>
+          <t>Rimborsi</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/transazioni-effettuate-con-strumenti-di-pagamento-elettronico</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rimborsi/</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>Comunicazioni</t>
-        </is>
-      </c>
-      <c r="E254" t="inlineStr">
-        <is>
-          <t>Comunicare le transazioni con pagamenti elettronici</t>
+          <t>ADER - Rimborsi</t>
         </is>
       </c>
       <c r="G254" t="inlineStr"/>
       <c r="H254" t="inlineStr"/>
       <c r="I254" t="inlineStr">
         <is>
-          <t>Richieste e comunicazioni all'Agenzia</t>
+          <t>Pagamenti e Rimborsi</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
         <is>
-          <t>Comunicazioni da parte di operatori finanziari</t>
-        </is>
-      </c>
-      <c r="N254" t="inlineStr">
-        <is>
-          <t>Comunicare le transazioni con pagamenti elettronici come operatore finanziario o gestore di sistemi di pagamento: trasmissione annuale dei dati sulle operazioni di pagamento elettronico per i controlli fiscali.</t>
+          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="n">
-        <v>486</v>
+        <v>404</v>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>Presentare la dichiarazione IVA in caso di fallimento (art. 74-bis)</t>
+          <t>Ricevere le notifiche di Agenzia delle Entrate-Riscossione a mezzo PEC</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/dichiarazione-iva-74-bis-2021</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/notifica-a-mezzo-pec/</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>Comunicazioni</t>
+          <t>ADER - Notifica a mezzo PEC</t>
         </is>
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>Presentare la dichiarazione IVA in caso di fallimento (art. 74-bis)</t>
+          <t>Ricevere le notifiche di Agenzia delle Entrate-Riscossione a mezzo PEC</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G255" t="inlineStr"/>
       <c r="H255" t="inlineStr"/>
       <c r="I255" t="inlineStr">
         <is>
-          <t>Aprire e gestire un'attività o Partita IVA</t>
+          <t>Richieste e comunicazioni all'Agenzia</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
         <is>
-          <t>Dichiarazioni imprese e società</t>
+          <t>Notifiche e domicilio digitale</t>
+        </is>
+      </c>
+      <c r="M255" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti ricorrenti</t>
+        </is>
+      </c>
+      <c r="N255" t="inlineStr">
+        <is>
+          <t>Ricevere le notifiche di cartelle e atti dell'Agenzia delle Entrate-Riscossione come contribuente titolare di PEC: modalità di notifica telematica, effetti, ricevute e gestione del domicilio digitale.</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="n">
-        <v>487</v>
+        <v>405</v>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>Imposta assicurazioni premi e accessori</t>
+          <t>Delegare un intermediario per la posizione debitoria in Agenzia delle Entrate-Riscossione</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/schede/dichiarazioni/denuncia-imposta-assicurazioni-2019</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/delega-un-intermediario/</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>Dichiarazioni</t>
+          <t>ADER - Home - Cittadini - Delega un intermediario</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>Delegare un intermediario per la posizione debitoria in Agenzia delle Entrate-Riscossione</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>Scheda istanza</t>
         </is>
       </c>
       <c r="G256" t="inlineStr"/>
       <c r="H256" t="inlineStr"/>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>Richieste e comunicazioni all'Agenzia</t>
+        </is>
+      </c>
+      <c r="K256" t="inlineStr">
+        <is>
+          <t>Deleghe e abilitazioni</t>
+        </is>
+      </c>
+      <c r="M256" t="inlineStr">
+        <is>
+          <t>Life events — Amministrazione fiscale</t>
+        </is>
+      </c>
+      <c r="N256" t="inlineStr">
+        <is>
+          <t>Delegare un intermediario (commercialista, CAF, avvocato) per la gestione della propria posizione debitoria in Agenzia delle Entrate-Riscossione come contribuente: consultazione cartelle, rateizzazioni, sospensioni e istanze.</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="n">
-        <v>488</v>
+        <v>406</v>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>Dichiarazione imposta di bollo assolta in modo virtuale</t>
+          <t>Operare come persona di fiducia o rappresentante presso Agenzia delle Entrate-Riscossione</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/schede/dichiarazioni/pagamento-virtuale-imposta-bollo</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/opera-come-persona-di-fiducia-o-rappresentante/</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>Dichiarazioni</t>
+          <t>ADER - Home - Cittadini - Opera come persona di fiducia o rappresentante</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>Operare come persona di fiducia o rappresentante presso Agenzia delle Entrate-Riscossione</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>Scheda istanza</t>
         </is>
       </c>
       <c r="G257" t="inlineStr"/>
       <c r="H257" t="inlineStr"/>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>Richieste e comunicazioni all'Agenzia</t>
+        </is>
+      </c>
+      <c r="K257" t="inlineStr">
+        <is>
+          <t>Deleghe e abilitazioni</t>
+        </is>
+      </c>
+      <c r="M257" t="inlineStr">
+        <is>
+          <t>Life events — Assistenza familiare</t>
+        </is>
+      </c>
+      <c r="N257" t="inlineStr">
+        <is>
+          <t>Operare come persona di fiducia o rappresentante di un contribuente presso Agenzia delle Entrate-Riscossione: gestire la posizione debitoria di un familiare, tutore o assistito autorizzato ai servizi.</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="n">
-        <v>489</v>
+        <v>411</v>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>ISA – Indici sintetici di affidabilità</t>
+          <t>Compensazioni crediti d'imposta</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/schede/dichiarazioni/isa-2020</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/imprese/Compensazioni/CompensazioniCreditiiDimposta/</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>Dichiarazioni</t>
+          <t>ADER - Compensazioni - Compensazioni crediti d'imposta</t>
         </is>
       </c>
       <c r="G258" t="inlineStr"/>
       <c r="H258" t="inlineStr"/>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>Pagamenti e Rimborsi</t>
+        </is>
+      </c>
+      <c r="K258" t="inlineStr">
+        <is>
+          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="n">
-        <v>490</v>
+        <v>412</v>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>Intra 12</t>
+          <t>Compensazioni con crediti verso la PA</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/schede/dichiarazioni/intra-12</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/imprese/Compensazioni/CompensazioniConCreditiVersoLaPA/</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>Dichiarazioni</t>
+          <t>ADER - Compensazioni - Compensazioni con crediti verso la PA</t>
         </is>
       </c>
       <c r="G259" t="inlineStr"/>
       <c r="H259" t="inlineStr"/>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>Pagamenti e Rimborsi</t>
+        </is>
+      </c>
+      <c r="K259" t="inlineStr">
+        <is>
+          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="n">
-        <v>491</v>
+        <v>429</v>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>Intra 13</t>
+          <t>Rimborsi in conto fiscale</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/schede/dichiarazioni/intra-13</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/imprese/Rimborsi/RimborsiInContoFiscale/</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>Dichiarazioni</t>
+          <t>ADER - Rimborsi - Rimborsi in conto fiscale</t>
         </is>
       </c>
       <c r="G260" t="inlineStr"/>
       <c r="H260" t="inlineStr"/>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>Pagamenti e Rimborsi</t>
+        </is>
+      </c>
+      <c r="K260" t="inlineStr">
+        <is>
+          <t>Richieste di rimborso</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="n">
-        <v>492</v>
+        <v>430</v>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>Elenchi riepilogativi (Intrastat)</t>
+          <t>Rimborsi IVA in conto fiscale</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/schede/dichiarazioni/elenchi-riepilogativi-intrastat</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/imprese/Rimborsi/RimborsiIvaInContoFiscale/</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>Dichiarazioni</t>
+          <t>ADER - Rimborsi - Rimborsi IVA in conto fiscale</t>
         </is>
       </c>
       <c r="G261" t="inlineStr"/>
       <c r="H261" t="inlineStr"/>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>Pagamenti e Rimborsi</t>
+        </is>
+      </c>
+      <c r="K261" t="inlineStr">
+        <is>
+          <t>Richieste di rimborso</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="n">
-        <v>493</v>
+        <v>431</v>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>Dichiarazione Iva 74-bis</t>
+          <t>Cessione - Revoca - Sospensione</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/schede/dichiarazioni/iva-74-bis</t>
+          <t>https://www.agenziaentrateriscossione.gov.it/it/imprese/Rimborsi/CessioneRevocaSospensioneRimborsi/</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>Dichiarazioni</t>
+          <t>ADER - Rimborsi - Cessione - Revoca - Sospensione</t>
         </is>
       </c>
       <c r="G262" t="inlineStr"/>
       <c r="H262" t="inlineStr"/>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>Pagamenti e Rimborsi</t>
+        </is>
+      </c>
+      <c r="K262" t="inlineStr">
+        <is>
+          <t>Richieste di rimborso</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="n">
-        <v>494</v>
+        <v>462</v>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>Scelte dell’8, 5 e 2 per mille Irpef 2026</t>
+          <t>Aderire al ravvedimento speciale CPB per le annualità 2019-2023</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/scelte-dell-8-5-e-2-per-mille-irpef-2026</t>
+          <t>https://www.agenziaentrate.gov.it/portale/ravvedimento-cpb-annualita-2019-2023</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>Dichiarazioni</t>
+          <t>Accertamenti e regolarizzazioni</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>Aderire al ravvedimento speciale CPB per le annualità 2019-2023</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G263" t="inlineStr"/>
       <c r="H263" t="inlineStr"/>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>Controlli fiscali e contenziosi</t>
+        </is>
+      </c>
+      <c r="K263" t="inlineStr">
+        <is>
+          <t>Controlli automatici</t>
+        </is>
+      </c>
+      <c r="M263" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti straordinari</t>
+        </is>
+      </c>
+      <c r="N263" t="inlineStr">
+        <is>
+          <t>Aderire al ravvedimento speciale collegato al Concordato Preventivo Biennale (CPB) come contribuente ISA: regolarizzare le annualità 2019-2023 pagando un'imposta sostitutiva ridotta.</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="n">
-        <v>495</v>
+        <v>464</v>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>Autodichiarazione requisiti Temporary framework</t>
+          <t>Aderire al ravvedimento speciale CPB per le annualità 2018-2022</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/autodichiarazione-requisiti-temporary-framework</t>
+          <t>https://www.agenziaentrate.gov.it/portale/ravvedimento-cpb</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>Dichiarazioni</t>
+          <t>Accertamenti e regolarizzazioni</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>Aderire al ravvedimento speciale CPB per le annualità 2018-2022</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G264" t="inlineStr"/>
       <c r="H264" t="inlineStr"/>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>Controlli fiscali e contenziosi</t>
+        </is>
+      </c>
+      <c r="K264" t="inlineStr">
+        <is>
+          <t>Controlli automatici</t>
+        </is>
+      </c>
+      <c r="M264" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti straordinari</t>
+        </is>
+      </c>
+      <c r="N264" t="inlineStr">
+        <is>
+          <t>Aderire al ravvedimento speciale collegato al Concordato Preventivo Biennale (CPB) come contribuente ISA: regolarizzare le annualità 2018-2022 pagando un'imposta sostitutiva ridotta.</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="n">
-        <v>496</v>
+        <v>466</v>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Irap 2026</t>
+          <t>Richiedere il credito d'imposta aggiuntivo per investimenti nella ZES unica 2025</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/dichiarazione-irap-2026</t>
+          <t>https://www.agenziaentrate.gov.it/portale/credito-d-imposta-aggiuntivo-zes-unica-2025</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>Dichiarazioni</t>
+          <t>Agevolazioni</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>Richiedere il credito d'imposta aggiuntivo per investimenti nella ZES unica 2025</t>
         </is>
       </c>
       <c r="G265" t="inlineStr"/>
       <c r="H265" t="inlineStr"/>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>Ottenere bonus e agevolazioni</t>
+        </is>
+      </c>
+      <c r="K265" t="inlineStr">
+        <is>
+          <t>Agevolazioni imprese e start-up</t>
+        </is>
+      </c>
+      <c r="M265" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Investimenti agevolati</t>
+        </is>
+      </c>
+      <c r="N265" t="inlineStr">
+        <is>
+          <t>Richiedere il credito d'imposta aggiuntivo per investimenti nella ZES unica del Mezzogiorno 2025 come impresa: agevolazione integrativa al credito ZES base, fruibile in compensazione tramite F24.</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="n">
-        <v>497</v>
+        <v>467</v>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Presentare documenti telematici per atti del debitore</t>
+          <t>Richiedere il credito d'imposta per cuochi professionisti</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/presentazione-telematica-documenti-corte-dei-conti-enti-e-pa</t>
+          <t>https://www.agenziaentrate.gov.it/portale/credito-di-imposta-per-cuochi-professionisti</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>FabbricatiTerreni</t>
+          <t>Agevolazioni</t>
         </is>
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>Presentare documenti telematici per atti del debitore</t>
-        </is>
-      </c>
-      <c r="F266" t="inlineStr">
-        <is>
-          <t>Servizio/Modello/Strumento</t>
+          <t>Richiedere il credito d'imposta per cuochi professionisti</t>
         </is>
       </c>
       <c r="G266" t="inlineStr"/>
       <c r="H266" t="inlineStr"/>
       <c r="I266" t="inlineStr">
         <is>
-          <t>Casa e terreni</t>
+          <t>Ottenere bonus e agevolazioni</t>
         </is>
       </c>
       <c r="K266" t="inlineStr">
         <is>
-          <t>Dati ipotecari e pubblicita' immobiliare</t>
-        </is>
-      </c>
-      <c r="M266" t="inlineStr">
-        <is>
-          <t>Starting a Small Claims Procedure — Contenzioso fiscale / Procedure legali</t>
+          <t>Agevolazioni imprese e start-up</t>
         </is>
       </c>
       <c r="N266" t="inlineStr">
         <is>
-          <t>Presentare documenti telematici per atti del debitore con impatto sui registri immobiliari come professionista: piattaforma per la trasmissione di atti relativi a procedure concorsuali e tutela dei creditori.</t>
+          <t>Richiedere il credito d'imposta per cuochi professionisti come lavoratore autonomo o dipendente del settore: agevolazione su acquisto strumenti professionali, fruibile tramite F24 in compensazione.</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="n">
-        <v>498</v>
+        <v>468</v>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Consultare il registro delle partite catastali</t>
+          <t>Richiedere il contributo a fondo perduto per interventi edilizi 2024</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/consultazione-registro-partite-catastali</t>
+          <t>https://www.agenziaentrate.gov.it/portale/contributo-a-fondo-perduto-per-interventi-edilizi-2024</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>FabbricatiTerreni</t>
+          <t>Agevolazioni</t>
         </is>
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>Consultare il registro delle partite catastali</t>
-        </is>
-      </c>
-      <c r="F267" t="inlineStr">
-        <is>
-          <t>Servizio/Modello/Strumento</t>
+          <t>Richiedere il contributo a fondo perduto per interventi edilizi 2024</t>
         </is>
       </c>
       <c r="G267" t="inlineStr"/>
       <c r="H267" t="inlineStr"/>
       <c r="I267" t="inlineStr">
         <is>
-          <t>Casa e terreni</t>
+          <t>Ottenere bonus e agevolazioni</t>
         </is>
       </c>
       <c r="K267" t="inlineStr">
         <is>
-          <t>Consultazione banche dati catastali</t>
+          <t>Agevolazioni casa e ristrutturazioni</t>
+        </is>
+      </c>
+      <c r="M267" t="inlineStr">
+        <is>
+          <t>Property purchase / renovation — Casa</t>
         </is>
       </c>
       <c r="N267" t="inlineStr">
         <is>
-          <t>Consultare il registro delle partite catastali come notaio o ricercatore: registro storico utile per ricostruire la successione dei passaggi di proprietà e degli accatastamenti di un immobile.</t>
+          <t>Richiedere il contributo a fondo perduto per interventi edilizi 2024 come proprietario o inquilino: sostegno economico per lavori di ristrutturazione con requisiti di reddito ISEE ridotto.</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="n">
-        <v>499</v>
+        <v>469</v>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Richiedere Codice Fiscale e Tessera Sanitaria</t>
+          <t>Ottenere le agevolazioni per il primo insediamento di imprese giovanili in agricoltura</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/codice-fiscale-e-tessera-sanitaria</t>
+          <t>https://www.agenziaentrate.gov.it/portale/primo-insediamento-delle-imprese-giovanili-in-agricoltura</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>Istanze</t>
+          <t>Agevolazioni</t>
         </is>
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Richiedere Codice Fiscale e Tessera Sanitaria</t>
-        </is>
-      </c>
-      <c r="F268" t="inlineStr">
-        <is>
-          <t>Scheda informativa</t>
+          <t>Ottenere le agevolazioni per il primo insediamento di imprese giovanili in agricoltura</t>
         </is>
       </c>
       <c r="G268" t="inlineStr"/>
       <c r="H268" t="inlineStr"/>
       <c r="I268" t="inlineStr">
         <is>
-          <t>Codice Fiscale e Tessera Sanitaria</t>
+          <t>Ottenere bonus e agevolazioni</t>
+        </is>
+      </c>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t>Aprire e gestire un'attività o Partita IVA</t>
+        </is>
+      </c>
+      <c r="K268" t="inlineStr">
+        <is>
+          <t>Agevolazioni imprese e start-up</t>
+        </is>
+      </c>
+      <c r="L268" t="inlineStr">
+        <is>
+          <t>Avviare un'attività</t>
+        </is>
+      </c>
+      <c r="N268" t="inlineStr">
+        <is>
+          <t>Ottenere le agevolazioni per il primo insediamento di imprenditori agricoli come giovane sotto i 41 anni: contributi e benefici fiscali sul reddito d'impresa per chi avvia un'attività agricola.</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="n">
-        <v>500</v>
+        <v>470</v>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Registrare la partita IVA italiana come soggetto non residente tramite rappresentante fiscale</t>
+          <t>Richiedere il credito d'imposta per la formazione in gestione agricola</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/registrazione-iva-per-soggetti-non-residenti-tramite-rappresentante-fiscale</t>
+          <t>https://www.agenziaentrate.gov.it/portale/credito-d-imposta-per-le-spese-sostenute-per-la-partecipazione-a-corsi-di-formazione-attinenti-alla-gestione-dell-azienda-agricola</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>Istanze</t>
+          <t>Agevolazioni</t>
         </is>
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>Registrare la partita IVA italiana come soggetto non residente tramite rappresentante fiscale</t>
-        </is>
-      </c>
-      <c r="F269" t="inlineStr">
-        <is>
-          <t>Scheda informativa</t>
+          <t>Richiedere il credito d'imposta per la formazione in gestione agricola</t>
         </is>
       </c>
       <c r="G269" t="inlineStr"/>
       <c r="H269" t="inlineStr"/>
       <c r="I269" t="inlineStr">
         <is>
-          <t>Fiscalità internazionale e residenti all'estero</t>
+          <t>Ottenere bonus e agevolazioni</t>
         </is>
       </c>
       <c r="K269" t="inlineStr">
         <is>
-          <t>Identificazione fiscale per non residenti</t>
-        </is>
-      </c>
-      <c r="M269" t="inlineStr">
-        <is>
-          <t>Business Start-Up — Avvio attività / Apertura P.IVA</t>
+          <t>Agevolazioni imprese e start-up</t>
         </is>
       </c>
       <c r="N269" t="inlineStr">
         <is>
-          <t>Procedura per la registrazione IVA di soggetti non residenti tramite nomina di un rappresentante fiscale in Italia.</t>
+          <t>Richiedere il credito d'imposta per la formazione in gestione d'impresa come imprenditore: agevolazione su corsi di alta formazione manageriale, fruibile in compensazione tramite F24.</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="n">
-        <v>501</v>
+        <v>472</v>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Operare come persona di fiducia o rappresentante presso la Riscossione</t>
+          <t>Iscriversi al contributo del 5 per mille</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/schede/istanze/domicilio-per-notifica-atti</t>
+          <t>https://www.agenziaentrate.gov.it/portale/contributo-del-5-per-mille-anno-2026</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>Istanze</t>
+          <t>Agevolazioni</t>
         </is>
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>Operare come persona di fiducia o rappresentante presso la Riscossione</t>
+          <t>Iscriversi al contributo del 5 per mille</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>Scheda complessa</t>
         </is>
       </c>
       <c r="G270" t="inlineStr"/>
       <c r="H270" t="inlineStr"/>
       <c r="I270" t="inlineStr">
         <is>
-          <t>Richieste e comunicazioni all'Agenzia</t>
+          <t>Ottenere bonus e agevolazioni</t>
         </is>
       </c>
       <c r="K270" t="inlineStr">
         <is>
-          <t>Notifiche e domicilio digitale</t>
+          <t>Enti del Terzo Settore</t>
         </is>
       </c>
       <c r="N270" t="inlineStr">
         <is>
-          <t>Operare come persona di fiducia o rappresentante presso l'Agenzia delle Entrate per conto di un altro contribuente: procedura per gestire pratiche fiscali, dichiarazioni e cassetto fiscale di un familiare o terzo delegante.</t>
+          <t>Iscriversi al contributo del 5 per mille come ente del Terzo Settore, ONLUS, associazione, ente di ricerca o altro soggetto ammesso: presentazione domanda e mantenimento dei requisiti per ricevere le quote IRPEF dei contribuenti.</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="n">
-        <v>502</v>
+        <v>474</v>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Verpflichtungen nach der Registrierung von Mietverträgen für Immobilien</t>
+          <t>Aderire al regime IVA transfrontaliero di franchigia</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/ted-adempimenti-successivi-registrazione-contratti-locazione-beni-immobili</t>
+          <t>https://www.agenziaentrate.gov.it/portale/nuovo-regime-iva-per-le-piccole-imprese</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>Registrazione contratti - atti</t>
+          <t>Agevolazioni</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Aderire al regime IVA transfrontaliero di franchigia</t>
         </is>
       </c>
       <c r="G271" t="inlineStr"/>
       <c r="H271" t="inlineStr"/>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>Ottenere bonus e agevolazioni</t>
+        </is>
+      </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>Fiscalità internazionale e residenti all'estero</t>
+        </is>
+      </c>
+      <c r="K271" t="inlineStr">
+        <is>
+          <t>Regimi opzionali per le imprese e professionisti</t>
+        </is>
+      </c>
+      <c r="L271" t="inlineStr">
+        <is>
+          <t>IVA e adempimenti</t>
+        </is>
+      </c>
+      <c r="N271" t="inlineStr">
+        <is>
+          <t>Aderire al regime IVA transfrontaliero di franchigia come piccola impresa: regime che esonera dall'addebito IVA negli altri Stati UE in cui si vendono beni o servizi, soglia di volume d'affari 100.000€ annui.</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="n">
-        <v>503</v>
+        <v>475</v>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Verbale di distribuzione utili – Modello RAP</t>
+          <t>Adottare il sistema di controllo del rischio fiscale</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/verbale-di-distribuzione-utili-modello-rap</t>
+          <t>https://www.agenziaentrate.gov.it/portale/regime-opzionale-di-adozione-del-sistema-di-controllo-del-rischio-fiscale</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>Registrazione contratti - atti</t>
+          <t>Agevolazioni</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>Adottare il sistema di controllo del rischio fiscale</t>
         </is>
       </c>
       <c r="G272" t="inlineStr"/>
       <c r="H272" t="inlineStr"/>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>Ottenere bonus e agevolazioni</t>
+        </is>
+      </c>
+      <c r="K272" t="inlineStr">
+        <is>
+          <t>Regimi opzionali per le imprese e professionisti</t>
+        </is>
+      </c>
+      <c r="N272" t="inlineStr">
+        <is>
+          <t>Adottare il sistema di controllo del rischio fiscale (Tax Control Framework, TCF) come grande impresa: insieme di procedure interne per identificare, misurare e gestire il rischio fiscale, requisito per la cooperative compliance.</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="n">
-        <v>504</v>
+        <v>476</v>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Compilare e inviare la dichiarazione fiscale Globe (Pillar Two)</t>
+          <t>Richiedere il credito d'imposta per investimenti nella ZES unica 2026</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/dichiarazione-fiscale-globe</t>
+          <t>https://www.agenziaentrate.gov.it/portale/credito-d-imposta-per-investimenti-nella-zes-unica-zes-2026-</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>Dichiarazioni</t>
+          <t>Agevolazioni</t>
         </is>
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>Compilare e inviare la dichiarazione fiscale Globe (Pillar Two)</t>
-        </is>
-      </c>
-      <c r="F273" t="inlineStr">
-        <is>
-          <t>Servizio/Modello/Strumento</t>
+          <t>Richiedere il credito d'imposta per investimenti nella ZES unica 2026</t>
         </is>
       </c>
       <c r="G273" t="inlineStr"/>
       <c r="H273" t="inlineStr"/>
       <c r="I273" t="inlineStr">
         <is>
-          <t>Compilare ed inviare dichiarazioni</t>
+          <t>Ottenere bonus e agevolazioni</t>
         </is>
       </c>
       <c r="K273" t="inlineStr">
         <is>
-          <t>Dichiarazioni imprese e societa'</t>
-        </is>
-      </c>
-      <c r="M273" t="inlineStr">
-        <is>
-          <t>Regular Business Operations — Gestione attività / Adempimenti ricorrenti</t>
+          <t>Agevolazioni imprese e start-up</t>
         </is>
       </c>
       <c r="N273" t="inlineStr">
         <is>
-          <t>Compilare e inviare la dichiarazione fiscale Globe (Pillar Two OCSE) come grande gruppo multinazionale: applicazione dell'aliquota minima del 15% sulle imposte effettive per giurisdizione, dichiarazione annuale.</t>
+          <t>Richiedere il credito d'imposta per investimenti nella ZES (Zona Economica Speciale) unica del Mezzogiorno come impresa (annualità 2026): agevolazione su beni strumentali nuovi, fruibile in compensazione tramite F24.</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="n">
-        <v>505</v>
+        <v>477</v>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Registrare un pegno mobiliare non possessorio</t>
+          <t>Richiedere il credito d'imposta per investimenti nelle ZLS 2026</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrate.gov.it/portale/pegno-mobiliare-non-possessorio</t>
+          <t>https://www.agenziaentrate.gov.it/portale/zls-2026</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>Istanze</t>
+          <t>Agevolazioni</t>
         </is>
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>Registrare un pegno mobiliare non possessorio</t>
-        </is>
-      </c>
-      <c r="F274" t="inlineStr">
-        <is>
-          <t>Servizio/Modello/Strumento</t>
+          <t>Richiedere il credito d'imposta per investimenti nelle ZLS 2026</t>
         </is>
       </c>
       <c r="G274" t="inlineStr"/>
       <c r="H274" t="inlineStr"/>
       <c r="I274" t="inlineStr">
         <is>
-          <t>Richieste e comunicazioni all'Agenzia</t>
+          <t>Ottenere bonus e agevolazioni</t>
         </is>
       </c>
       <c r="K274" t="inlineStr">
         <is>
-          <t>Altre dichiarazioni e comunicazioni</t>
-        </is>
-      </c>
-      <c r="M274" t="inlineStr">
-        <is>
-          <t>Regular Business Operations — Gestione attività / Adempimenti ricorrenti</t>
+          <t>Agevolazioni imprese e start-up</t>
         </is>
       </c>
       <c r="N274" t="inlineStr">
         <is>
-          <t>Registrare un pegno mobiliare non possessorio come impresa creditrice: garanzia reale su beni mobili senza spossessamento del debitore, iscritta nel registro telematico tenuto dall'Agenzia delle Entrate.</t>
+          <t>Richiedere il credito d'imposta per investimenti nelle aree del Centro Italia colpite dal sisma come impresa: agevolazione fiscale per ripresa economica, fruibile in compensazione tramite F24.</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="n">
-        <v>384</v>
+        <v>478</v>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Pagamenti</t>
+          <t>Comunicare il regime IVA transfrontaliero di franchigia</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Pagamenti/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/comunicazione-trimestrale-del-regime-transfrontaliero-di-franchigia</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>ADER - Pagamenti</t>
+          <t>Comunicazioni</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Comunicare il regime IVA transfrontaliero di franchigia</t>
         </is>
       </c>
       <c r="G275" t="inlineStr"/>
       <c r="H275" t="inlineStr"/>
       <c r="I275" t="inlineStr">
         <is>
-          <t>Pagamenti e Rimborsi</t>
+          <t>Aprire e gestire un'attività o Partita IVA</t>
+        </is>
+      </c>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>Fiscalità internazionale e residenti all'estero</t>
         </is>
       </c>
       <c r="K275" t="inlineStr">
         <is>
-          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
+          <t>Guida IVA per imprese e professionisti</t>
+        </is>
+      </c>
+      <c r="L275" t="inlineStr">
+        <is>
+          <t>IVA e adempimenti</t>
+        </is>
+      </c>
+      <c r="N275" t="inlineStr">
+        <is>
+          <t>Comunicare l'adesione al regime IVA transfrontaliero di franchigia come piccola impresa: adempimento obbligatorio per beneficiare dell'esonero IVA negli altri Stati UE, con monitoraggio della soglia 100.000€.</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="n">
-        <v>385</v>
+        <v>479</v>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Come e dove pagare</t>
+          <t>Optare per il regime IVA per servizi di trasporto e logistica</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Pagamenti/comedovepagare/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/opzione-per-le-prestazioni-di-servizi-rese-nei-confronti-di-imprese-che-svolgono-attivita-di-trasporto-movimentazione-merci-e-servizi-di-logistica</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>ADER - Pagamenti - Come e dove pagare</t>
+          <t>Comunicazioni</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>Optare per il regime IVA per servizi di trasporto e logistica</t>
         </is>
       </c>
       <c r="G276" t="inlineStr"/>
       <c r="H276" t="inlineStr"/>
       <c r="I276" t="inlineStr">
         <is>
-          <t>Pagamenti e Rimborsi</t>
+          <t>Aprire e gestire un'attività o Partita IVA</t>
         </is>
       </c>
       <c r="K276" t="inlineStr">
         <is>
-          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
+          <t>Guida IVA per imprese e professionisti</t>
+        </is>
+      </c>
+      <c r="N276" t="inlineStr">
+        <is>
+          <t>Optare per il regime IVA dedicato ai servizi di trasporto e logistica internazionale come impresa del settore: regole specifiche su esenzioni e applicazione dell'IVA nei trasporti intra-UE ed extra-UE.</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="n">
-        <v>386</v>
+        <v>480</v>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Pagamenti dall'estero</t>
+          <t>Comunicare le spese sanitarie sostenute</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Pagamenti/PagamentiDallEstero/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/spese-sanitarie</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>ADER - Pagamenti - Pagamenti dall'estero</t>
+          <t>Comunicazioni</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Comunicare le spese sanitarie sostenute</t>
         </is>
       </c>
       <c r="G277" t="inlineStr"/>
       <c r="H277" t="inlineStr"/>
       <c r="I277" t="inlineStr">
         <is>
-          <t>Pagamenti e Rimborsi</t>
-        </is>
-      </c>
-      <c r="J277" t="inlineStr">
-        <is>
-          <t>Fiscalità internazionale e residenti all'estero</t>
+          <t>Compilare ed inviare dichiarazioni</t>
         </is>
       </c>
       <c r="K277" t="inlineStr">
         <is>
-          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
-        </is>
-      </c>
-      <c r="M277" t="inlineStr">
-        <is>
-          <t>Regular Business Operations — Gestione attività / Adempimenti ricorrenti</t>
+          <t>Dati per la dichiarazione precompilata</t>
         </is>
       </c>
       <c r="N277" t="inlineStr">
         <is>
-          <t>Servizio per cittadini residenti all'estero per pagare cartelle e avvisi tramite pagoPA, bonifico bancario o canali telematici.</t>
+          <t>Comunicare le spese sanitarie sostenute dai cittadini come struttura sanitaria, farmacia, medico o altro operatore: trasmissione al Sistema TS (Tessera Sanitaria) per la dichiarazione precompilata e la detrazione IRPEF.</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="n">
-        <v>387</v>
+        <v>481</v>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Compensazioni</t>
+          <t>Comunicare i proventi dalla cessione di energia da fonti rinnovabili</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Compensazioni/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/com_impianto_alimentato_fonti_derivabili</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>ADER - Compensazioni</t>
+          <t>Comunicazioni</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>Comunicare i proventi dalla cessione di energia da fonti rinnovabili</t>
         </is>
       </c>
       <c r="G278" t="inlineStr"/>
       <c r="H278" t="inlineStr"/>
       <c r="I278" t="inlineStr">
         <is>
-          <t>Pagamenti e Rimborsi</t>
+          <t>Compilare ed inviare dichiarazioni</t>
         </is>
       </c>
       <c r="K278" t="inlineStr">
         <is>
-          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
+          <t>Dati per la dichiarazione precompilata</t>
+        </is>
+      </c>
+      <c r="N278" t="inlineStr">
+        <is>
+          <t>Comunicare i proventi dalla cessione di energia da fonti rinnovabili come gestore di impianto fotovoltaico, eolico o biomasse: trasmissione annuale al GSE e all'Agenzia ai fini fiscali.</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="n">
-        <v>388</v>
+        <v>482</v>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Rateizzazione</t>
+          <t>Indicare il domicilio digitale (PEC) per ricevere atti e comunicazioni</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rateizzazione/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/comunicazione-del-domicilio-digitale-speciale</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>ADER - Rateizzazione</t>
+          <t>Comunicazioni</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>Indicare il domicilio digitale (PEC) per ricevere atti e comunicazioni</t>
         </is>
       </c>
       <c r="G279" t="inlineStr"/>
       <c r="H279" t="inlineStr"/>
       <c r="I279" t="inlineStr">
         <is>
-          <t>Pagamenti e Rimborsi</t>
+          <t>Richieste e comunicazioni all'Agenzia</t>
         </is>
       </c>
       <c r="K279" t="inlineStr">
         <is>
-          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
+          <t>Notifiche e domicilio digitale</t>
+        </is>
+      </c>
+      <c r="N279" t="inlineStr">
+        <is>
+          <t>Indicare il domicilio digitale (PEC, Posta Elettronica Certificata) per ricevere atti dall'Agenzia delle Entrate: comunicazione che permette notifica telematica di accertamenti, comunicazioni e provvedimenti.</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="n">
-        <v>389</v>
+        <v>483</v>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t xml:space="preserve"> La  rateizzazione dal 1° gennaio 2025</t>
+          <t>Delegare l'accesso ai servizi online dell'Agenzia delle Entrate e della Riscossione</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rateizzazione/la-rateizzazione/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/delega-unica-ai-servizi-on-line-dell-agenzia-delle-entrate-e-dell-agenzia-delle-entrate-riscossione</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>ADER - Rateizzazione - La rateizzazione dal 1° gennaio 2025</t>
+          <t>Comunicazioni</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Delegare l'accesso ai servizi online dell'Agenzia delle Entrate e della Riscossione</t>
         </is>
       </c>
       <c r="G280" t="inlineStr"/>
       <c r="H280" t="inlineStr"/>
       <c r="I280" t="inlineStr">
         <is>
-          <t>Pagamenti e Rimborsi</t>
+          <t>Richieste e comunicazioni all'Agenzia</t>
         </is>
       </c>
       <c r="K280" t="inlineStr">
         <is>
-          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
+          <t>Deleghe e abilitazioni</t>
+        </is>
+      </c>
+      <c r="N280" t="inlineStr">
+        <is>
+          <t>Delegare l'accesso ai servizi online dell'Agenzia delle Entrate a un familiare, professionista o intermediario: procedura per autorizzare un terzo a operare sul proprio cassetto fiscale e dichiarazioni.</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="n">
-        <v>390</v>
+        <v>484</v>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Istanze "a semplice richiesta"</t>
+          <t>Comunicare la cessazione dell'incarico di depositario delle scritture contabili</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rateizzazione/istanze-a-semplice-richiesta/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/comunicazione-di-cessazione-incarico-di-depositario-scritture-contabili</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>ADER - Rateizzazione - Istanze "a semplice richiesta"</t>
+          <t>Comunicazioni</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Comunicare la cessazione dell'incarico di depositario delle scritture contabili</t>
         </is>
       </c>
       <c r="G281" t="inlineStr"/>
       <c r="H281" t="inlineStr"/>
       <c r="I281" t="inlineStr">
         <is>
-          <t>Pagamenti e Rimborsi</t>
+          <t>Aprire e gestire un'attività o Partita IVA</t>
         </is>
       </c>
       <c r="K281" t="inlineStr">
         <is>
-          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
+          <t>Avviare un'attività</t>
+        </is>
+      </c>
+      <c r="N281" t="inlineStr">
+        <is>
+          <t>Comunicare la cessazione dell'incarico come depositario delle scritture contabili: adempimento obbligatorio entro 30 giorni dalla rinuncia o revoca, comunicazione tramite modello AA9/12.</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="n">
-        <v>391</v>
+        <v>485</v>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Istanze "documentate"</t>
+          <t>Comunicare le transazioni con pagamenti elettronici</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rateizzazione/istanze-documentate/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/transazioni-effettuate-con-strumenti-di-pagamento-elettronico</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>ADER - Rateizzazione - Istanze "documentate"</t>
+          <t>Comunicazioni</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>Comunicare le transazioni con pagamenti elettronici</t>
         </is>
       </c>
       <c r="G282" t="inlineStr"/>
       <c r="H282" t="inlineStr"/>
       <c r="I282" t="inlineStr">
         <is>
-          <t>Pagamenti e Rimborsi</t>
+          <t>Richieste e comunicazioni all'Agenzia</t>
         </is>
       </c>
       <c r="K282" t="inlineStr">
         <is>
-          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
+          <t>Comunicazioni da parte di operatori finanziari</t>
+        </is>
+      </c>
+      <c r="N282" t="inlineStr">
+        <is>
+          <t>Comunicare le transazioni con pagamenti elettronici come operatore finanziario o gestore di sistemi di pagamento: trasmissione annuale dei dati sulle operazioni di pagamento elettronico per i controlli fiscali.</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="n">
-        <v>392</v>
+        <v>486</v>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Proroga del piano di rateizzazione</t>
+          <t>Presentare la dichiarazione IVA in caso di fallimento (art. 74-bis)</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rateizzazione/Proroga/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/dichiarazione-iva-74-bis-2021</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>ADER - Rateizzazione - Proroga del piano di rateizzazione</t>
+          <t>Comunicazioni</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>Presentare la dichiarazione IVA in caso di fallimento (art. 74-bis)</t>
         </is>
       </c>
       <c r="G283" t="inlineStr"/>
       <c r="H283" t="inlineStr"/>
       <c r="I283" t="inlineStr">
         <is>
-          <t>Pagamenti e Rimborsi</t>
+          <t>Compilare ed inviare dichiarazioni</t>
         </is>
       </c>
       <c r="K283" t="inlineStr">
         <is>
-          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
+          <t>Dichiarazioni imprese e societa'</t>
+        </is>
+      </c>
+      <c r="M283" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti straordinari</t>
+        </is>
+      </c>
+      <c r="N283" t="inlineStr">
+        <is>
+          <t>Presentare la dichiarazione IVA 74-bis 2021 come curatore fallimentare o commissario liquidatore: comunicare le operazioni IVA effettuate fino all'apertura della procedura concorsuale nel 2021.</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="n">
-        <v>393</v>
+        <v>487</v>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Istanze "documentate" - Indicatori</t>
+          <t>Denunciare l'imposta sulle assicurazioni, premi e accessori</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rateizzazione/istanze-documentate-indicatori/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/schede/dichiarazioni/denuncia-imposta-assicurazioni-2019</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>ADER - Rateizzazione - Istanze "documentate" - Indicatori</t>
+          <t>Dichiarazioni</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>Denunciare l'imposta sulle assicurazioni, premi e accessori</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G284" t="inlineStr"/>
       <c r="H284" t="inlineStr"/>
       <c r="I284" t="inlineStr">
         <is>
-          <t>Pagamenti e Rimborsi</t>
+          <t>Compilare ed inviare dichiarazioni</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
         <is>
-          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
+          <t>Dichiarazioni imprese e societa'</t>
+        </is>
+      </c>
+      <c r="M284" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti annuali</t>
+        </is>
+      </c>
+      <c r="N284" t="inlineStr">
+        <is>
+          <t>Denunciare l'imposta sulle assicurazioni, premi e accessori come compagnia assicurativa: dichiarazione annuale dei premi incassati soggetti a imposta secondo la Legge 1216/1961.</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="n">
-        <v>394</v>
+        <v>488</v>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Istanze "documentate" - Simula il numero delle rate</t>
+          <t>Presentare la dichiarazione dell'imposta di bollo assolta in modo virtuale</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rateizzazione/istanze-documentate-simula-il-numero-delle-rate/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/schede/dichiarazioni/pagamento-virtuale-imposta-bollo</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>ADER - Rateizzazione - Istanze "documentate" - Simula il numero delle rate</t>
+          <t>Dichiarazioni</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>Presentare la dichiarazione dell'imposta di bollo assolta in modo virtuale</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G285" t="inlineStr"/>
       <c r="H285" t="inlineStr"/>
       <c r="I285" t="inlineStr">
         <is>
-          <t>Pagamenti e Rimborsi</t>
+          <t>Compilare ed inviare dichiarazioni</t>
         </is>
       </c>
       <c r="K285" t="inlineStr">
         <is>
-          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
+          <t>Dichiarazioni imprese e societa'</t>
+        </is>
+      </c>
+      <c r="M285" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti annuali</t>
+        </is>
+      </c>
+      <c r="N285" t="inlineStr">
+        <is>
+          <t>Presentare la dichiarazione annuale dell'imposta di bollo assolta in modo virtuale come banca, ente autorizzato o notaio: riepilogo dei documenti soggetti a bollo virtuale nell'anno precedente.</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="n">
-        <v>395</v>
+        <v>489</v>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Cosa succede con la presentazione della richiesta di rateizzazione</t>
+          <t>Compilare gli Indici Sintetici di Affidabilità (ISA) per il proprio settore</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rateizzazione/cosa-succede-con-la-presentazione-della-richiesta-di-rateizzazione/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/schede/dichiarazioni/isa-2020</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>ADER - Rateizzazione - Cosa succede con la presentazione della richiesta</t>
+          <t>Dichiarazioni</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>Compilare gli Indici Sintetici di Affidabilità (ISA) per il proprio settore</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G286" t="inlineStr"/>
       <c r="H286" t="inlineStr"/>
       <c r="I286" t="inlineStr">
         <is>
-          <t>Pagamenti e Rimborsi</t>
+          <t>Compilare ed inviare dichiarazioni</t>
         </is>
       </c>
       <c r="K286" t="inlineStr">
         <is>
-          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
+          <t>Dichiarazioni imprese e societa'</t>
+        </is>
+      </c>
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti annuali</t>
+        </is>
+      </c>
+      <c r="N286" t="inlineStr">
+        <is>
+          <t>Compilare gli Indici Sintetici di Affidabilità Fiscale (ISA) 2026 come impresa o professionista: misurare il grado di affidabilità fiscale ottenendo un punteggio da 1 a 10, con eventuali benefici premiali.</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="n">
-        <v>396</v>
+        <v>490</v>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Decadenza dal piano di rateizzazione</t>
+          <t>Presentare il modello Intra 12 per acquisti intracomunitari da parte di enti non commerciali</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rateizzazione/decadenza-dal-piano-di-rateizzazione/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/schede/dichiarazioni/intra-12</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>ADER - Rateizzazione - Decadenza dal piano di rateizzazione</t>
+          <t>Dichiarazioni</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>Presentare il modello Intra 12 per acquisti intracomunitari da parte di enti non commerciali</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G287" t="inlineStr"/>
       <c r="H287" t="inlineStr"/>
       <c r="I287" t="inlineStr">
         <is>
-          <t>Pagamenti e Rimborsi</t>
+          <t>Compilare ed inviare dichiarazioni</t>
         </is>
       </c>
       <c r="K287" t="inlineStr">
         <is>
-          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
+          <t>Dichiarazioni imprese e societa'</t>
+        </is>
+      </c>
+      <c r="M287" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti mensili</t>
+        </is>
+      </c>
+      <c r="N287" t="inlineStr">
+        <is>
+          <t>Presentare il modello Intra 12 come ente non commerciale o agricoltore forfetario: dichiarare gli acquisti intracomunitari di beni e servizi non soggetti al regime IVA ordinario.</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="n">
-        <v>397</v>
+        <v>491</v>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Rateizzazione - Domiciliazione bancaria</t>
+          <t>Presentare il modello Intra 13 per acquisti intracomunitari</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rateizzazione/rateizzazione-domiciliazione-bancaria/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/schede/dichiarazioni/intra-13</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>ADER - Rateizzazione - Domiciliazione bancaria</t>
+          <t>Dichiarazioni</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>Presentare il modello Intra 13 per acquisti intracomunitari</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G288" t="inlineStr"/>
       <c r="H288" t="inlineStr"/>
       <c r="I288" t="inlineStr">
         <is>
-          <t>Pagamenti e Rimborsi</t>
+          <t>Compilare ed inviare dichiarazioni</t>
         </is>
       </c>
       <c r="K288" t="inlineStr">
         <is>
-          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
+          <t>Dichiarazioni imprese e societa'</t>
+        </is>
+      </c>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti mensili</t>
+        </is>
+      </c>
+      <c r="N288" t="inlineStr">
+        <is>
+          <t>Presentare il modello Intra 13 come ente non commerciale o produttore agricolo: dichiarare gli acquisti intracomunitari sotto la soglia di rilevanza IVA da parte di soggetti particolari.</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="n">
-        <v>398</v>
+        <v>492</v>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Rateizzazione - Richiedi i moduli di pagamento</t>
+          <t>Presentare gli elenchi riepilogativi Intrastat delle operazioni con l'estero UE</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rateizzazione/bollettini-moduli-di-pagamento/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/schede/dichiarazioni/elenchi-riepilogativi-intrastat</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>ADER - Rateizzazione - Richiedi i moduli di pagamento</t>
+          <t>Dichiarazioni</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>Presentare gli elenchi riepilogativi Intrastat delle operazioni con l'estero UE</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G289" t="inlineStr"/>
       <c r="H289" t="inlineStr"/>
       <c r="I289" t="inlineStr">
         <is>
-          <t>Pagamenti e Rimborsi</t>
+          <t>Compilare ed inviare dichiarazioni</t>
         </is>
       </c>
       <c r="K289" t="inlineStr">
         <is>
-          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
+          <t>Dichiarazioni imprese e societa'</t>
+        </is>
+      </c>
+      <c r="M289" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti periodici</t>
+        </is>
+      </c>
+      <c r="N289" t="inlineStr">
+        <is>
+          <t>Presentare gli elenchi riepilogativi Intrastat come impresa che effettua operazioni intracomunitarie: comunicare vendite, acquisti e prestazioni di servizi verso/da paesi UE con frequenza mensile o trimestrale.</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="n">
-        <v>399</v>
+        <v>493</v>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Enti che rateizzano in proprio e tributi/tipi imposta non rateizzabili</t>
+          <t>Presentare la dichiarazione IVA 74-bis in caso di procedura concorsuale</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rateizzazione/EntiCheRateizzanoInProprioETributiNonRateizzabili/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/schede/dichiarazioni/iva-74-bis</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>ADER - Rateizzazione - Enti che rateizzano in proprio</t>
+          <t>Dichiarazioni</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>Presentare la dichiarazione IVA 74-bis in caso di procedura concorsuale</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G290" t="inlineStr"/>
       <c r="H290" t="inlineStr"/>
       <c r="I290" t="inlineStr">
         <is>
-          <t>Pagamenti e Rimborsi</t>
+          <t>Compilare ed inviare dichiarazioni</t>
         </is>
       </c>
       <c r="K290" t="inlineStr">
         <is>
-          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
+          <t>Dichiarazioni imprese e societa'</t>
+        </is>
+      </c>
+      <c r="M290" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti straordinari</t>
+        </is>
+      </c>
+      <c r="N290" t="inlineStr">
+        <is>
+          <t>Presentare la dichiarazione IVA 74-bis come curatore fallimentare o commissario liquidatore: comunicare le operazioni IVA effettuate fino all'apertura della procedura concorsuale del contribuente.</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="n">
-        <v>400</v>
+        <v>494</v>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Enti che hanno autorizzato l’Agente della riscossione a concedere la rateizzazione</t>
+          <t>Destinare l'8, il 5 e il 2 per mille dell'IRPEF nella dichiarazione 2026</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rateizzazione/Enti-Rateizzazione/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/scelte-dell-8-5-e-2-per-mille-irpef-2026</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>ADER - Rateizzazione - Enti autorizzati alla riscossione</t>
+          <t>Dichiarazioni</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>Destinare l'8, il 5 e il 2 per mille dell'IRPEF nella dichiarazione 2026</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G291" t="inlineStr"/>
       <c r="H291" t="inlineStr"/>
       <c r="I291" t="inlineStr">
         <is>
-          <t>Pagamenti e Rimborsi</t>
+          <t>Compilare ed inviare dichiarazioni</t>
         </is>
       </c>
       <c r="K291" t="inlineStr">
         <is>
-          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
+          <t>Dichiarazione dei redditi (730, Redditi PF)</t>
+        </is>
+      </c>
+      <c r="M291" t="inlineStr">
+        <is>
+          <t>Life events — Dichiarazione dei redditi</t>
+        </is>
+      </c>
+      <c r="N291" t="inlineStr">
+        <is>
+          <t>Destinare l'8, il 5 e il 2 per mille dell'IRPEF come cittadino nella dichiarazione dei redditi 2026: scegliere la confessione religiosa, l'ente del Terzo Settore o il partito politico a cui destinare le quote.</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="n">
-        <v>401</v>
+        <v>495</v>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Sospensione</t>
+          <t>Presentare l'autodichiarazione dei requisiti Temporary Framework (aiuti Covid)</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Sospensione/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/autodichiarazione-requisiti-temporary-framework</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>ADER - Sospensione</t>
+          <t>Dichiarazioni</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>Presentare l'autodichiarazione dei requisiti Temporary Framework (aiuti Covid)</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G292" t="inlineStr"/>
       <c r="H292" t="inlineStr"/>
       <c r="I292" t="inlineStr">
         <is>
-          <t>Pagamenti e Rimborsi</t>
+          <t>Compilare ed inviare dichiarazioni</t>
         </is>
       </c>
       <c r="K292" t="inlineStr">
         <is>
-          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
+          <t>Dichiarazioni imprese e societa'</t>
+        </is>
+      </c>
+      <c r="M292" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti straordinari</t>
+        </is>
+      </c>
+      <c r="N292" t="inlineStr">
+        <is>
+          <t>Presentare l'autodichiarazione dei requisiti Temporary Framework come impresa beneficiaria di aiuti Covid-19: attestare il rispetto dei massimali europei sugli aiuti ricevuti durante l'emergenza.</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="n">
-        <v>402</v>
+        <v>496</v>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Annullamento del debito</t>
+          <t>Presentare la dichiarazione IRAP 2026 come impresa o ente</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/AnnullamentoDelDebito/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/dichiarazione-irap-2026</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>ADER - Annullamento del debito</t>
+          <t>Dichiarazioni</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>Presentare la dichiarazione IRAP 2026 come impresa o ente</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G293" t="inlineStr"/>
       <c r="H293" t="inlineStr"/>
       <c r="I293" t="inlineStr">
         <is>
-          <t>Pagamenti e Rimborsi</t>
+          <t>Compilare ed inviare dichiarazioni</t>
         </is>
       </c>
       <c r="K293" t="inlineStr">
         <is>
-          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
+          <t>Dichiarazioni imprese e societa'</t>
+        </is>
+      </c>
+      <c r="M293" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti annuali</t>
+        </is>
+      </c>
+      <c r="N293" t="inlineStr">
+        <is>
+          <t>Presentare la dichiarazione IRAP 2026 come impresa, professionista o ente: liquidare l'imposta regionale sulle attività produttive dovuta per l'anno d'imposta 2025.</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="n">
-        <v>403</v>
+        <v>497</v>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Rimborsi</t>
+          <t>Presentare documenti telematici per atti del debitore</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/Rimborsi/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/presentazione-telematica-documenti-corte-dei-conti-enti-e-pa</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>ADER - Rimborsi</t>
+          <t>FabbricatiTerreni</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>Presentare documenti telematici per atti del debitore</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>Servizio/Modello/Strumento</t>
         </is>
       </c>
       <c r="G294" t="inlineStr"/>
       <c r="H294" t="inlineStr"/>
       <c r="I294" t="inlineStr">
         <is>
-          <t>Pagamenti e Rimborsi</t>
+          <t>Casa e terreni</t>
         </is>
       </c>
       <c r="K294" t="inlineStr">
         <is>
-          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
+          <t>Dati ipotecari e pubblicita' immobiliare</t>
+        </is>
+      </c>
+      <c r="M294" t="inlineStr">
+        <is>
+          <t>Starting a Small Claims Procedure — Contenzioso fiscale / Procedure legali</t>
+        </is>
+      </c>
+      <c r="N294" t="inlineStr">
+        <is>
+          <t>Presentare documenti telematici per atti del debitore con impatto sui registri immobiliari come professionista: piattaforma per la trasmissione di atti relativi a procedure concorsuali e tutela dei creditori.</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="n">
-        <v>404</v>
+        <v>498</v>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Notifica a mezzo PEC</t>
+          <t>Consultare il registro delle partite catastali</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/notifica-a-mezzo-pec/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/consultazione-registro-partite-catastali</t>
         </is>
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>ADER - Notifica a mezzo PEC</t>
+          <t>FabbricatiTerreni</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>Consultare il registro delle partite catastali</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>Servizio/Modello/Strumento</t>
         </is>
       </c>
       <c r="G295" t="inlineStr"/>
       <c r="H295" t="inlineStr"/>
       <c r="I295" t="inlineStr">
         <is>
-          <t>Richieste e comunicazioni all'Agenzia</t>
+          <t>Casa e terreni</t>
         </is>
       </c>
       <c r="K295" t="inlineStr">
         <is>
-          <t>Notifiche e domicilio digitale</t>
+          <t>Consultazione banche dati catastali</t>
+        </is>
+      </c>
+      <c r="N295" t="inlineStr">
+        <is>
+          <t>Consultare il registro delle partite catastali come notaio o ricercatore: registro storico utile per ricostruire la successione dei passaggi di proprietà e degli accatastamenti di un immobile.</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="n">
-        <v>405</v>
+        <v>499</v>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Delega un intermediario</t>
+          <t>Richiedere Codice Fiscale e Tessera Sanitaria</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/delega-un-intermediario/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/codice-fiscale-e-tessera-sanitaria</t>
         </is>
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>ADER - Home - Cittadini - Delega un intermediario</t>
+          <t>Istanze</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>Richiedere Codice Fiscale e Tessera Sanitaria</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G296" t="inlineStr"/>
       <c r="H296" t="inlineStr"/>
       <c r="I296" t="inlineStr">
         <is>
-          <t>Controlli fiscali e contenziosi</t>
+          <t>Codice Fiscale e Tessera Sanitaria</t>
+        </is>
+      </c>
+      <c r="K296" t="inlineStr">
+        <is>
+          <t>Identificativi fiscali e abilitazioni</t>
+        </is>
+      </c>
+      <c r="M296" t="inlineStr">
+        <is>
+          <t>Life events — Identità e residenza</t>
+        </is>
+      </c>
+      <c r="N296" t="inlineStr">
+        <is>
+          <t>Richiedere il codice fiscale e la tessera sanitaria come cittadino italiano o straniero residente in Italia: identificativo fiscale univoco necessario per lavorare, aprire un conto, avere accesso al SSN.</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="n">
-        <v>406</v>
+        <v>500</v>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Opera come persona di fiducia o rappresentante</t>
+          <t>Registrare la partita IVA italiana come soggetto non residente tramite rappresentante fiscale</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/cittadini/opera-come-persona-di-fiducia-o-rappresentante/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/registrazione-iva-per-soggetti-non-residenti-tramite-rappresentante-fiscale</t>
         </is>
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>ADER - Home - Cittadini - Opera come persona di fiducia o rappresentante</t>
+          <t>Istanze</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Registrare la partita IVA italiana come soggetto non residente tramite rappresentante fiscale</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Scheda informativa</t>
         </is>
       </c>
       <c r="G297" t="inlineStr"/>
       <c r="H297" t="inlineStr"/>
       <c r="I297" t="inlineStr">
         <is>
-          <t>Controlli fiscali e contenziosi</t>
+          <t>Fiscalità internazionale e residenti all'estero</t>
+        </is>
+      </c>
+      <c r="K297" t="inlineStr">
+        <is>
+          <t>Identificazione fiscale per non residenti</t>
+        </is>
+      </c>
+      <c r="M297" t="inlineStr">
+        <is>
+          <t>Business Start-Up — Avvio attività / Apertura P.IVA</t>
+        </is>
+      </c>
+      <c r="N297" t="inlineStr">
+        <is>
+          <t>Procedura per la registrazione IVA di soggetti non residenti tramite nomina di un rappresentante fiscale in Italia.</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="n">
-        <v>411</v>
+        <v>501</v>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Compensazioni crediti d'imposta</t>
+          <t>Operare come persona di fiducia o rappresentante presso la Riscossione</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/imprese/Compensazioni/CompensazioniCreditiiDimposta/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/schede/istanze/domicilio-per-notifica-atti</t>
         </is>
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>ADER - Compensazioni - Compensazioni crediti d'imposta</t>
+          <t>Istanze</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>Operare come persona di fiducia o rappresentante presso la Riscossione</t>
         </is>
       </c>
       <c r="G298" t="inlineStr"/>
       <c r="H298" t="inlineStr"/>
       <c r="I298" t="inlineStr">
         <is>
-          <t>Pagamenti e Rimborsi</t>
+          <t>Richieste e comunicazioni all'Agenzia</t>
         </is>
       </c>
       <c r="K298" t="inlineStr">
         <is>
-          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
+          <t>Notifiche e domicilio digitale</t>
+        </is>
+      </c>
+      <c r="N298" t="inlineStr">
+        <is>
+          <t>Operare come persona di fiducia o rappresentante presso l'Agenzia delle Entrate per conto di un altro contribuente: procedura per gestire pratiche fiscali, dichiarazioni e cassetto fiscale di un familiare o terzo delegante.</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="n">
-        <v>412</v>
+        <v>502</v>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Compensazioni con crediti verso la PA</t>
+          <t>Comunicare gli adempimenti successivi alla registrazione di un contratto di locazione (in lingua tedesca)</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/imprese/Compensazioni/CompensazioniConCreditiVersoLaPA/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/ted-adempimenti-successivi-registrazione-contratti-locazione-beni-immobili</t>
         </is>
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>ADER - Compensazioni - Compensazioni con crediti verso la PA</t>
+          <t>Registrazione contratti - atti</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>Comunicare gli adempimenti successivi alla registrazione di un contratto di locazione (in lingua tedesca)</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>Scheda istanza</t>
         </is>
       </c>
       <c r="G299" t="inlineStr"/>
       <c r="H299" t="inlineStr"/>
       <c r="I299" t="inlineStr">
         <is>
-          <t>Pagamenti e Rimborsi</t>
+          <t>Casa e terreni</t>
         </is>
       </c>
       <c r="K299" t="inlineStr">
         <is>
-          <t>Pagamenti all'Agenzia delle Entrate-Riscossione</t>
+          <t>Affitti e locazioni</t>
+        </is>
+      </c>
+      <c r="M299" t="inlineStr">
+        <is>
+          <t>Property purchase / renovation — Affitto</t>
+        </is>
+      </c>
+      <c r="N299" t="inlineStr">
+        <is>
+          <t>Comunicare gli adempimenti successivi alla registrazione di un contratto di locazione come locatore in Alto Adige: proroghe, cessioni, risoluzioni anticipate — versione bilingue italiano-tedesco.</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="n">
-        <v>429</v>
+        <v>503</v>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Rimborsi in conto fiscale</t>
+          <t>Registrare il verbale di distribuzione utili con il modello RAP</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/imprese/Rimborsi/RimborsiInContoFiscale/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/verbale-di-distribuzione-utili-modello-rap</t>
         </is>
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>ADER - Rimborsi - Rimborsi in conto fiscale</t>
+          <t>Registrazione contratti - atti</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>Registrare il verbale di distribuzione utili con il modello RAP</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>Scheda istanza</t>
         </is>
       </c>
       <c r="G300" t="inlineStr"/>
       <c r="H300" t="inlineStr"/>
       <c r="I300" t="inlineStr">
         <is>
-          <t>Pagamenti e Rimborsi</t>
+          <t>Compilare ed inviare dichiarazioni</t>
         </is>
       </c>
       <c r="K300" t="inlineStr">
         <is>
-          <t>Richieste di rimborso</t>
+          <t>Dichiarazioni imprese e societa'</t>
+        </is>
+      </c>
+      <c r="M300" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Adempimenti straordinari</t>
+        </is>
+      </c>
+      <c r="N300" t="inlineStr">
+        <is>
+          <t>Registrare il verbale di distribuzione utili come società di capitali tramite il modello RAP (Registrazione Atti Privati): trasmettere telematicamente il verbale assembleare di distribuzione dividendi.</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="n">
-        <v>430</v>
+        <v>504</v>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Rimborsi IVA in conto fiscale</t>
+          <t>Compilare e inviare la dichiarazione fiscale Globe (Pillar Two)</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/imprese/Rimborsi/RimborsiIvaInContoFiscale/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/dichiarazione-fiscale-globe</t>
         </is>
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>ADER - Rimborsi - Rimborsi IVA in conto fiscale</t>
+          <t>Dichiarazioni</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>Compilare e inviare la dichiarazione fiscale Globe (Pillar Two)</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>Servizio/Modello/Strumento</t>
         </is>
       </c>
       <c r="G301" t="inlineStr"/>
       <c r="H301" t="inlineStr"/>
       <c r="I301" t="inlineStr">
         <is>
-          <t>Pagamenti e Rimborsi</t>
+          <t>Compilare ed inviare dichiarazioni</t>
         </is>
       </c>
       <c r="K301" t="inlineStr">
         <is>
-          <t>Richieste di rimborso</t>
+          <t>Dichiarazioni imprese e societa'</t>
+        </is>
+      </c>
+      <c r="M301" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Gestione attività / Adempimenti ricorrenti</t>
+        </is>
+      </c>
+      <c r="N301" t="inlineStr">
+        <is>
+          <t>Compilare e inviare la dichiarazione fiscale Globe (Pillar Two OCSE) come grande gruppo multinazionale: applicazione dell'aliquota minima del 15% sulle imposte effettive per giurisdizione, dichiarazione annuale.</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="n">
-        <v>431</v>
+        <v>505</v>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Cessione - Revoca - Sospensione</t>
+          <t>Registrare un pegno mobiliare non possessorio</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>https://www.agenziaentrateriscossione.gov.it/it/imprese/Rimborsi/CessioneRevocaSospensioneRimborsi/</t>
+          <t>https://www.agenziaentrate.gov.it/portale/pegno-mobiliare-non-possessorio</t>
         </is>
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>ADER - Rimborsi - Cessione - Revoca - Sospensione</t>
+          <t>Istanze</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>Registrare un pegno mobiliare non possessorio</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>Servizio/Modello/Strumento</t>
         </is>
       </c>
       <c r="G302" t="inlineStr"/>
       <c r="H302" t="inlineStr"/>
       <c r="I302" t="inlineStr">
         <is>
-          <t>Pagamenti e Rimborsi</t>
+          <t>Richieste e comunicazioni all'Agenzia</t>
         </is>
       </c>
       <c r="K302" t="inlineStr">
         <is>
-          <t>Richieste di rimborso</t>
+          <t>Altre dichiarazioni e comunicazioni</t>
+        </is>
+      </c>
+      <c r="M302" t="inlineStr">
+        <is>
+          <t>Regular Business Operations — Gestione attività / Adempimenti ricorrenti</t>
+        </is>
+      </c>
+      <c r="N302" t="inlineStr">
+        <is>
+          <t>Registrare un pegno mobiliare non possessorio come impresa creditrice: garanzia reale su beni mobili senza spossessamento del debitore, iscritta nel registro telematico tenuto dall'Agenzia delle Entrate.</t>
         </is>
       </c>
     </row>

</xml_diff>